<commit_message>
Atualiza dados de pedidos e vendedores com novas entradas
</commit_message>
<xml_diff>
--- a/nao_positivados_07-2026.xlsx
+++ b/nao_positivados_07-2026.xlsx
@@ -22237,468 +22237,471 @@
     <t>VINHO BAROLO BUSSIA RISERVA 750ML</t>
   </si>
   <si>
+    <t>VINHO TINTO BURDIZZO APPASSIMENTO 750ML</t>
+  </si>
+  <si>
+    <t>WHISKY BUCHANANS 12 YEARS 1L</t>
+  </si>
+  <si>
+    <t>JIM BEAM BLACK CHERRY 1L</t>
+  </si>
+  <si>
+    <t>WHISKY BALLANTINE S SUNSHINE 700ML</t>
+  </si>
+  <si>
+    <t>WHISKY JACK DANIELS 1L - DEST</t>
+  </si>
+  <si>
+    <t>WHISKY JACK DANIELS APPLE 1L - DEST</t>
+  </si>
+  <si>
+    <t>AGUARDENTE OLD CESAR 88 965 ML</t>
+  </si>
+  <si>
+    <t>WHISKEY JACK DANIELS HONEY 1 L</t>
+  </si>
+  <si>
+    <t>RUM BACARDI GOLD 980ML</t>
+  </si>
+  <si>
+    <t>WHISKY JIM BEAM HONEY 1L</t>
+  </si>
+  <si>
+    <t>CATUABA SELVAGEM 900ML</t>
+  </si>
+  <si>
+    <t>WHISKY JACK DANIELS APPLE 1L</t>
+  </si>
+  <si>
+    <t>VODKA ABSOLUT RASPBERRY - 750ML</t>
+  </si>
+  <si>
+    <t>CACHACA SELETA PRATA 1L</t>
+  </si>
+  <si>
+    <t>APERITIVO CAMPARI 998ML</t>
+  </si>
+  <si>
+    <t>CONHAQUE DREHER 900ML</t>
+  </si>
+  <si>
+    <t>LICOR STOCK COCONUT 720 ML</t>
+  </si>
+  <si>
+    <t>SMIRNOFF ICE 24X275ML LONG</t>
+  </si>
+  <si>
+    <t>WHISKY BALLANTINE S FINEST 750ML</t>
+  </si>
+  <si>
+    <t>WHISKY JAMESON CASKMATES IPA 750ML</t>
+  </si>
+  <si>
+    <t>WHISKY PASSPORT APPLE 670ML</t>
+  </si>
+  <si>
+    <t>VODKA SMIRNOFF 600 ML</t>
+  </si>
+  <si>
+    <t>LICOR BALLENA COCO 750ML</t>
+  </si>
+  <si>
+    <t>GIN ROCKS GREEN APPLE 1LT</t>
+  </si>
+  <si>
+    <t>GIN BEEFEATER BOTANICS 750ML</t>
+  </si>
+  <si>
+    <t>CHANDON PASSION ROSE 750ML</t>
+  </si>
+  <si>
+    <t>WHISKY WHITE HORSE - 1L</t>
+  </si>
+  <si>
+    <t>WHISKY J WALKER RED LABEL 1L</t>
+  </si>
+  <si>
+    <t>WHISKY J WALKER BLACK LABEL 1L</t>
+  </si>
+  <si>
+    <t>CHANDON PASSION ON ICE 750 ML</t>
+  </si>
+  <si>
+    <t>VINHO ARESTI ESTATE S. CAB SAUV 750ML</t>
+  </si>
+  <si>
+    <t>RC ATUM PEDACOS EM OLEO 24X140G</t>
+  </si>
+  <si>
+    <t>RED BULL TROPICAL 24X250ML</t>
+  </si>
+  <si>
+    <t>AMARULA C LIQUEUR 750 ML + 1 COPO</t>
+  </si>
+  <si>
+    <t>SABOR DO SABOR GIN + COMBO MELANCIA</t>
+  </si>
+  <si>
+    <t>CERVEJA HEINEKEN 473ML (LATAO) - 12 UNID</t>
+  </si>
+  <si>
+    <t>REFRESCO DE UVA MINECRAFT 24X200ML</t>
+  </si>
+  <si>
+    <t>LICOR CAN FIREBALL CX C/ 6X50ML</t>
+  </si>
+  <si>
+    <t>STEINHAGER LOEWE 960ML</t>
+  </si>
+  <si>
+    <t>RUM BACARDI SUPERIOR 980ML</t>
+  </si>
+  <si>
+    <t>VILLA ROSA BRANCO 750ML</t>
+  </si>
+  <si>
+    <t>SMIRNOFF RED PET 1750 ML</t>
+  </si>
+  <si>
+    <t>CERVEJA AMSTEL ULTRA 473 ML</t>
+  </si>
+  <si>
+    <t>ICE 51 LIMAO LONG NECK 24X275ML</t>
+  </si>
+  <si>
+    <t>LICOR COINTREAU 700 ML</t>
+  </si>
+  <si>
+    <t>CERVEJA AMSTEL PURO MALTE 473 ML</t>
+  </si>
+  <si>
+    <t>VINHO CASA PERINI CHARDONNAY 750ML</t>
+  </si>
+  <si>
+    <t>GIN ROCKS WATERMELON 1000ML</t>
+  </si>
+  <si>
+    <t>CERVEJA AMSTEL LAGER 0,269LT SHR 12UNPBR</t>
+  </si>
+  <si>
+    <t>CERVEJA HEINEKEN - KEG 5 LITROS C/2 DESC</t>
+  </si>
+  <si>
+    <t>BALA HALLS EXTRA FORTE C/21 UND</t>
+  </si>
+  <si>
+    <t>CHICLETE TRIDENT MORANGO C/21 UN</t>
+  </si>
+  <si>
+    <t>NG BARRA NEUGE 80G CROCANTE (DP 16X80G)</t>
+  </si>
+  <si>
+    <t>NG BARRA NEUGE 80G BRANCO (DP 16X80G)</t>
+  </si>
+  <si>
+    <t>GIN MARINA 750ML</t>
+  </si>
+  <si>
+    <t>NG BARRA 80G 40% MEIO AMARGO (DP 16X80G)</t>
+  </si>
+  <si>
+    <t>RED BULL SF MAÇA 24X250ML</t>
+  </si>
+  <si>
+    <t>RANCHEIRO RECHEADO CHOCOLATE 90G</t>
+  </si>
+  <si>
+    <t>JACK DANIELS HONEY 1 L</t>
+  </si>
+  <si>
+    <t>ST PIERRE LATA MARGARITA LT 6X270ML</t>
+  </si>
+  <si>
+    <t>NG AMOR CARIOCA BOMBOM 200G (10X20G)</t>
+  </si>
+  <si>
+    <t>ST PIERRE LATA SUGAR FREE LT 24X270ML</t>
+  </si>
+  <si>
+    <t>WHISKY GENTLEMAN JACK 1L</t>
+  </si>
+  <si>
+    <t>ST PIERRE ZERO LATA TROPICAL LT 6X310ML</t>
+  </si>
+  <si>
+    <t>4 PACK RED BULL SUGAR FREE</t>
+  </si>
+  <si>
+    <t>CHICLETE TRIDENT MENTA C/21 UN</t>
+  </si>
+  <si>
+    <t>ST PIERRE ZERO LATA COLA LT 6X310ML</t>
+  </si>
+  <si>
+    <t>NG BARRA NEUGE 80G COOKIES BRANCO (DP 16</t>
+  </si>
+  <si>
+    <t>NG BARRA NEUGE 80G AO LEITE (DP 16X80G)</t>
+  </si>
+  <si>
+    <t>ST PIERRE LATA RED MINT LT 24X270ML</t>
+  </si>
+  <si>
+    <t>WHISKY JACK DANIELS 700ML - DEST</t>
+  </si>
+  <si>
+    <t>WHISKY WHITE HORSE - 500ML</t>
+  </si>
+  <si>
+    <t>WHISKY BUCHANANS 12 YEARS 750ML</t>
+  </si>
+  <si>
+    <t>4 PACK RED BULL MORANGO PESSEGO</t>
+  </si>
+  <si>
+    <t>MARTINI RISERVA RUBINO 750 ML</t>
+  </si>
+  <si>
+    <t>WHISKY CHIVAS XV GOLD 700ML</t>
+  </si>
+  <si>
+    <t>VILLA ROSA COLHEITA TINTO  750ML</t>
+  </si>
+  <si>
+    <t>TEQUILA DON JULIO BLANCO 750ML</t>
+  </si>
+  <si>
+    <t>CHAMPAGNE RUINART BLANC DE BLANCS 750ML</t>
+  </si>
+  <si>
+    <t>RC ATUM PEDACOS MOLHO DE TOMATE 24X140G</t>
+  </si>
+  <si>
+    <t>NAVEIA ORIGINAL 12X1L</t>
+  </si>
+  <si>
+    <t>NAVEIA BARISTA 12X1L</t>
+  </si>
+  <si>
+    <t>PINATI SIMPLE WHEY CARAM. SALGADO 16X35G</t>
+  </si>
+  <si>
+    <t>XAROPE FABBRI AMARENA 560ML</t>
+  </si>
+  <si>
+    <t>RC PATE ATUM COM AZEITONAS 12X80G</t>
+  </si>
+  <si>
+    <t>RC SARDINHA EM OLEO 125G</t>
+  </si>
+  <si>
+    <t>RUM BACARDI SUPERIOR 700ML</t>
+  </si>
+  <si>
+    <t>LICOR BALLENA MORANGO 750 ML</t>
+  </si>
+  <si>
+    <t>DP DADINHO BITZ AO LEITE 105G</t>
+  </si>
+  <si>
+    <t>PINATI NUTS COCO 16X4X25G</t>
+  </si>
+  <si>
+    <t>MARTINI ROSATO 750 ML</t>
+  </si>
+  <si>
+    <t>PINATI NUTS ZERO ORIGINAL 16X4X25G</t>
+  </si>
+  <si>
+    <t>PINATI NUTS ORIGINAL 16X4X30G</t>
+  </si>
+  <si>
+    <t>PINATI SLIM WHEY BEIJINHO 16X35G</t>
+  </si>
+  <si>
+    <t>PINATI DB WHEY AVELA E LEITE 12X50G</t>
+  </si>
+  <si>
+    <t>PINATI DOUBLE BAR BRIGADEIRO 32X35G</t>
+  </si>
+  <si>
+    <t>RC ATUM RALADO OLEO 24X140G</t>
+  </si>
+  <si>
+    <t>PINATI SLIM WHEY BRIGADEIRO 16X35G</t>
+  </si>
+  <si>
+    <t>4 PACK RED BULL SF AMORA</t>
+  </si>
+  <si>
+    <t>PIRASSUNUNGA 51 965 ML</t>
+  </si>
+  <si>
+    <t>ESPUMANTE ALUD BRANCO 750ML</t>
+  </si>
+  <si>
+    <t>WHISKY J WALKER GOLD LABEL RESERVE 750ML</t>
+  </si>
+  <si>
+    <t>AMARULA C LIQUEUR 750 ML</t>
+  </si>
+  <si>
+    <t>CHICLETE TRIDENT FRESH HERBAL C/21 UN</t>
+  </si>
+  <si>
+    <t>RC SARDINHA 125G OLEO (05 UND)</t>
+  </si>
+  <si>
+    <t>NG NEUGEBAUER HITS 200G BOMBOM SORTIDO</t>
+  </si>
+  <si>
+    <t>BALA HALLS UVA VERDE C/21 UND</t>
+  </si>
+  <si>
+    <t>DP PACOCA DADINHO ZERO 24X18G</t>
+  </si>
+  <si>
+    <t>VEUVE CLICQUOT BRUT 750 ML</t>
+  </si>
+  <si>
+    <t>PACOCA GAMADINHO 100X15G</t>
+  </si>
+  <si>
+    <t>BOM AR AERO 360 ML ALEGRIA</t>
+  </si>
+  <si>
+    <t>CHICLETE TRIDENT HORTELA C/21 UN</t>
+  </si>
+  <si>
+    <t>AZEITE  ESSENZA D'ITALIA PREMIUM 5L</t>
+  </si>
+  <si>
+    <t>NG AMOR CARIOCA BOMBOM 200G BRANCO</t>
+  </si>
+  <si>
+    <t>RC ATUM RALADO MOLHO DE TOMATE 170G</t>
+  </si>
+  <si>
+    <t>CHICLETE TRIDENT MAX  HORTELA C/21 UN</t>
+  </si>
+  <si>
+    <t>CHICLETE TRIDENT MENTA C/ 14 UND</t>
+  </si>
+  <si>
+    <t>ST PIERRE ZERO LATA GREEN APPLE 24X310ML</t>
+  </si>
+  <si>
+    <t>CHICLETE TRIDENT MELANCIA C/21 UN</t>
+  </si>
+  <si>
+    <t>VINHO GRAVEDAD CARMENERE 750ML</t>
+  </si>
+  <si>
+    <t>NG AMOR CARIOCA BOMBOM BRANCO 500G</t>
+  </si>
+  <si>
+    <t>NG AMOR CARIOCA 200GR DUO (DP10 X20G)</t>
+  </si>
+  <si>
+    <t>WHISKY JIM BEAM RYE 700ML</t>
+  </si>
+  <si>
+    <t>CHICLETE TRIDENT MELANCIA C/ 14 UND</t>
+  </si>
+  <si>
+    <t>BOM AR AERO 360 ML CHEIRO DE TALCO</t>
+  </si>
+  <si>
+    <t>INSETICIDA SBP 360 ML ULTRA BARREIRA</t>
+  </si>
+  <si>
+    <t>4 PACK RED BULL SF BLUEBERRY BAUNILHA</t>
+  </si>
+  <si>
+    <t>4 PACK RED BULL SF NECTARINA 4X250ML</t>
+  </si>
+  <si>
+    <t>APERITIVO APEROL 750 ML</t>
+  </si>
+  <si>
+    <t>XAROPE MONIN MACA VERDE (APPLE) 700 ML</t>
+  </si>
+  <si>
+    <t>RED BULL SF NECTARINA 24X250ML</t>
+  </si>
+  <si>
+    <t>WHISKY J WALKER GREEN LABEL - 750ML</t>
+  </si>
+  <si>
+    <t>AGUA MINERAL MAMBA WATER C/ GAS 12X350ML</t>
+  </si>
+  <si>
+    <t>RED BULL CEREJA 24X250ML</t>
+  </si>
+  <si>
+    <t>AGUA NA LATA C/ GAS 12X310ML</t>
+  </si>
+  <si>
+    <t>XAROPE CHERRY MARIE BRIZARD 700ML</t>
+  </si>
+  <si>
+    <t>AGUA MINERAL MINALBA S/GAS LATA 12X310ML</t>
+  </si>
+  <si>
+    <t>VINHO ARESTI RESERVA CARMENERE 750ML</t>
+  </si>
+  <si>
+    <t>CERVEJA HEINEKEN ZERO LONG  24X330ML</t>
+  </si>
+  <si>
+    <t>VINHO HORIZONTE TINTO 750ML</t>
+  </si>
+  <si>
+    <t>LICOR CAN FIREBALL 750ML</t>
+  </si>
+  <si>
+    <t>FRISANTE MACAW TROPICAL MOSC. ROSE 750ML</t>
+  </si>
+  <si>
+    <t>FRISANTE MACAW TROPICAL MOSCATO 750ML</t>
+  </si>
+  <si>
+    <t>AGUA MINERAL MAMBA WATER S/ GAS 12X350ML</t>
+  </si>
+  <si>
+    <t>GIN INVICTUS MELANCIA 900ML</t>
+  </si>
+  <si>
+    <t>ESPUMANTE ARESTI CHARDONNAY 187,5ML</t>
+  </si>
+  <si>
+    <t>VINHO ARESTI ESTATE S. CARMENERE 750ML</t>
+  </si>
+  <si>
+    <t>TEQUILA EL JIMADOR REPOSADO 750 ML</t>
+  </si>
+  <si>
+    <t>NOSSO CHOP RED DRAFT VD 6X600ML</t>
+  </si>
+  <si>
+    <t>DRYCAT LONDON DRY GIN</t>
+  </si>
+  <si>
+    <t>GIN GORDONS PINK 700ML</t>
+  </si>
+  <si>
+    <t>VINHO ARESTI ESTATE S. CHARDONNAY 187ML</t>
+  </si>
+  <si>
+    <t>VINHO CAVAS DE ORO MALBEC 750ML</t>
+  </si>
+  <si>
+    <t>LICOR BANANINHA CARIOCA 750ML</t>
+  </si>
+  <si>
     <t>HUMB. CANALE DENARIO RESERVA CAB. FRANC</t>
   </si>
   <si>
-    <t>WHISKY BUCHANANS 12 YEARS 1L</t>
-  </si>
-  <si>
-    <t>JIM BEAM BLACK CHERRY 1L</t>
-  </si>
-  <si>
-    <t>WHISKY BALLANTINE S SUNSHINE 700ML</t>
-  </si>
-  <si>
-    <t>WHISKY JACK DANIELS 1L - DEST</t>
-  </si>
-  <si>
-    <t>WHISKY JACK DANIELS APPLE 1L - DEST</t>
-  </si>
-  <si>
-    <t>AGUARDENTE OLD CESAR 88 965 ML</t>
-  </si>
-  <si>
-    <t>WHISKEY JACK DANIELS HONEY 1 L</t>
-  </si>
-  <si>
-    <t>RUM BACARDI GOLD 980ML</t>
-  </si>
-  <si>
-    <t>WHISKY JIM BEAM HONEY 1L</t>
-  </si>
-  <si>
-    <t>CATUABA SELVAGEM 900ML</t>
-  </si>
-  <si>
-    <t>WHISKY JACK DANIELS APPLE 1L</t>
-  </si>
-  <si>
-    <t>VODKA ABSOLUT RASPBERRY - 750ML</t>
-  </si>
-  <si>
-    <t>CACHACA SELETA PRATA 1L</t>
-  </si>
-  <si>
-    <t>APERITIVO CAMPARI 998ML</t>
-  </si>
-  <si>
-    <t>CONHAQUE DREHER 900ML</t>
-  </si>
-  <si>
-    <t>LICOR STOCK COCONUT 720 ML</t>
-  </si>
-  <si>
-    <t>SMIRNOFF ICE 24X275ML LONG</t>
-  </si>
-  <si>
-    <t>WHISKY BALLANTINE S FINEST 750ML</t>
-  </si>
-  <si>
-    <t>WHISKY JAMESON CASKMATES IPA 750ML</t>
-  </si>
-  <si>
-    <t>WHISKY PASSPORT APPLE 670ML</t>
-  </si>
-  <si>
-    <t>VODKA SMIRNOFF 600 ML</t>
-  </si>
-  <si>
-    <t>LICOR BALLENA COCO 750ML</t>
-  </si>
-  <si>
-    <t>GIN ROCKS GREEN APPLE 1LT</t>
-  </si>
-  <si>
-    <t>GIN BEEFEATER BOTANICS 750ML</t>
-  </si>
-  <si>
-    <t>CHANDON PASSION ROSE 750ML</t>
-  </si>
-  <si>
-    <t>WHISKY WHITE HORSE - 1L</t>
-  </si>
-  <si>
-    <t>WHISKY J WALKER RED LABEL 1L</t>
-  </si>
-  <si>
-    <t>WHISKY J WALKER BLACK LABEL 1L</t>
-  </si>
-  <si>
-    <t>CHANDON PASSION ON ICE 750 ML</t>
-  </si>
-  <si>
-    <t>VINHO ARESTI ESTATE S. CAB SAUV 750ML</t>
-  </si>
-  <si>
-    <t>RC ATUM PEDACOS EM OLEO 24X140G</t>
-  </si>
-  <si>
-    <t>RED BULL TROPICAL 24X250ML</t>
-  </si>
-  <si>
-    <t>AMARULA C LIQUEUR 750 ML + 1 COPO</t>
-  </si>
-  <si>
-    <t>SABOR DO SABOR GIN + COMBO MELANCIA</t>
-  </si>
-  <si>
-    <t>CERVEJA HEINEKEN 473ML (LATAO) - 12 UNID</t>
-  </si>
-  <si>
-    <t>REFRESCO DE UVA MINECRAFT 24X200ML</t>
-  </si>
-  <si>
-    <t>LICOR CAN FIREBALL CX C/ 6X50ML</t>
-  </si>
-  <si>
-    <t>STEINHAGER LOEWE 960ML</t>
-  </si>
-  <si>
-    <t>RUM BACARDI SUPERIOR 980ML</t>
-  </si>
-  <si>
-    <t>VILLA ROSA BRANCO 750ML</t>
-  </si>
-  <si>
-    <t>SMIRNOFF RED PET 1750 ML</t>
-  </si>
-  <si>
-    <t>CERVEJA AMSTEL ULTRA 473 ML</t>
-  </si>
-  <si>
-    <t>ICE 51 LIMAO LONG NECK 24X275ML</t>
-  </si>
-  <si>
-    <t>LICOR COINTREAU 700 ML</t>
-  </si>
-  <si>
-    <t>CERVEJA AMSTEL PURO MALTE 473 ML</t>
-  </si>
-  <si>
-    <t>VINHO CASA PERINI CHARDONNAY 750ML</t>
-  </si>
-  <si>
-    <t>GIN ROCKS WATERMELON 1000ML</t>
-  </si>
-  <si>
-    <t>CERVEJA AMSTEL LAGER 0,269LT SHR 12UNPBR</t>
-  </si>
-  <si>
-    <t>CERVEJA HEINEKEN - KEG 5 LITROS C/2 DESC</t>
-  </si>
-  <si>
-    <t>BALA HALLS EXTRA FORTE C/21 UND</t>
-  </si>
-  <si>
-    <t>CHICLETE TRIDENT MORANGO C/21 UN</t>
-  </si>
-  <si>
-    <t>NG BARRA NEUGE 80G CROCANTE (DP 16X80G)</t>
-  </si>
-  <si>
-    <t>NG BARRA NEUGE 80G BRANCO (DP 16X80G)</t>
-  </si>
-  <si>
-    <t>GIN MARINA 750ML</t>
-  </si>
-  <si>
-    <t>NG BARRA 80G 40% MEIO AMARGO (DP 16X80G)</t>
-  </si>
-  <si>
-    <t>RED BULL SF MAÇA 24X250ML</t>
-  </si>
-  <si>
-    <t>RANCHEIRO RECHEADO CHOCOLATE 90G</t>
-  </si>
-  <si>
-    <t>JACK DANIELS HONEY 1 L</t>
-  </si>
-  <si>
-    <t>ST PIERRE LATA MARGARITA LT 6X270ML</t>
-  </si>
-  <si>
-    <t>NG AMOR CARIOCA BOMBOM 200G (10X20G)</t>
-  </si>
-  <si>
-    <t>ST PIERRE LATA SUGAR FREE LT 24X270ML</t>
-  </si>
-  <si>
-    <t>WHISKY GENTLEMAN JACK 1L</t>
-  </si>
-  <si>
-    <t>ST PIERRE ZERO LATA TROPICAL LT 6X310ML</t>
-  </si>
-  <si>
-    <t>4 PACK RED BULL SUGAR FREE</t>
-  </si>
-  <si>
-    <t>CHICLETE TRIDENT MENTA C/21 UN</t>
-  </si>
-  <si>
-    <t>ST PIERRE ZERO LATA COLA LT 6X310ML</t>
-  </si>
-  <si>
-    <t>NG BARRA NEUGE 80G COOKIES BRANCO (DP 16</t>
-  </si>
-  <si>
-    <t>NG BARRA NEUGE 80G AO LEITE (DP 16X80G)</t>
-  </si>
-  <si>
-    <t>ST PIERRE LATA RED MINT LT 24X270ML</t>
-  </si>
-  <si>
-    <t>WHISKY JACK DANIELS 700ML - DEST</t>
-  </si>
-  <si>
-    <t>WHISKY WHITE HORSE - 500ML</t>
-  </si>
-  <si>
-    <t>WHISKY BUCHANANS 12 YEARS 750ML</t>
-  </si>
-  <si>
-    <t>4 PACK RED BULL MORANGO PESSEGO</t>
-  </si>
-  <si>
-    <t>MARTINI RISERVA RUBINO 750 ML</t>
-  </si>
-  <si>
-    <t>WHISKY CHIVAS XV GOLD 700ML</t>
-  </si>
-  <si>
-    <t>VILLA ROSA COLHEITA TINTO  750ML</t>
-  </si>
-  <si>
-    <t>TEQUILA DON JULIO BLANCO 750ML</t>
-  </si>
-  <si>
-    <t>CHAMPAGNE RUINART BLANC DE BLANCS 750ML</t>
-  </si>
-  <si>
-    <t>RC ATUM PEDACOS MOLHO DE TOMATE 24X140G</t>
-  </si>
-  <si>
-    <t>NAVEIA ORIGINAL 12X1L</t>
-  </si>
-  <si>
-    <t>NAVEIA BARISTA 12X1L</t>
-  </si>
-  <si>
-    <t>PINATI SIMPLE WHEY CARAM. SALGADO 16X35G</t>
-  </si>
-  <si>
-    <t>XAROPE FABBRI AMARENA 560ML</t>
-  </si>
-  <si>
-    <t>RC PATE ATUM COM AZEITONAS 12X80G</t>
-  </si>
-  <si>
-    <t>RC SARDINHA EM OLEO 125G</t>
-  </si>
-  <si>
-    <t>RUM BACARDI SUPERIOR 700ML</t>
-  </si>
-  <si>
-    <t>LICOR BALLENA MORANGO 750 ML</t>
-  </si>
-  <si>
-    <t>DP DADINHO BITZ AO LEITE 105G</t>
-  </si>
-  <si>
-    <t>PINATI NUTS COCO 16X4X25G</t>
-  </si>
-  <si>
-    <t>MARTINI ROSATO 750 ML</t>
-  </si>
-  <si>
-    <t>PINATI NUTS ZERO ORIGINAL 16X4X25G</t>
-  </si>
-  <si>
-    <t>PINATI NUTS ORIGINAL 16X4X30G</t>
-  </si>
-  <si>
-    <t>PINATI SLIM WHEY BEIJINHO 16X35G</t>
-  </si>
-  <si>
-    <t>PINATI DB WHEY AVELA E LEITE 12X50G</t>
-  </si>
-  <si>
-    <t>PINATI DOUBLE BAR BRIGADEIRO 32X35G</t>
-  </si>
-  <si>
-    <t>RC ATUM RALADO OLEO 24X140G</t>
-  </si>
-  <si>
-    <t>PINATI SLIM WHEY BRIGADEIRO 16X35G</t>
-  </si>
-  <si>
-    <t>4 PACK RED BULL SF AMORA</t>
-  </si>
-  <si>
-    <t>PIRASSUNUNGA 51 965 ML</t>
-  </si>
-  <si>
-    <t>ESPUMANTE ALUD BRANCO 750ML</t>
-  </si>
-  <si>
-    <t>WHISKY J WALKER GOLD LABEL RESERVE 750ML</t>
-  </si>
-  <si>
-    <t>AMARULA C LIQUEUR 750 ML</t>
-  </si>
-  <si>
-    <t>CHICLETE TRIDENT FRESH HERBAL C/21 UN</t>
-  </si>
-  <si>
-    <t>RC SARDINHA 125G OLEO (05 UND)</t>
-  </si>
-  <si>
-    <t>NG NEUGEBAUER HITS 200G BOMBOM SORTIDO</t>
-  </si>
-  <si>
-    <t>BALA HALLS UVA VERDE C/21 UND</t>
-  </si>
-  <si>
-    <t>DP PACOCA DADINHO ZERO 24X18G</t>
-  </si>
-  <si>
-    <t>VEUVE CLICQUOT BRUT 750 ML</t>
-  </si>
-  <si>
-    <t>PACOCA GAMADINHO 100X15G</t>
-  </si>
-  <si>
-    <t>BOM AR AERO 360 ML ALEGRIA</t>
-  </si>
-  <si>
-    <t>CHICLETE TRIDENT HORTELA C/21 UN</t>
-  </si>
-  <si>
-    <t>AZEITE  ESSENZA D'ITALIA PREMIUM 5L</t>
-  </si>
-  <si>
-    <t>NG AMOR CARIOCA BOMBOM 200G BRANCO</t>
-  </si>
-  <si>
-    <t>RC ATUM RALADO MOLHO DE TOMATE 170G</t>
-  </si>
-  <si>
-    <t>CHICLETE TRIDENT MAX  HORTELA C/21 UN</t>
-  </si>
-  <si>
-    <t>CHICLETE TRIDENT MENTA C/ 14 UND</t>
-  </si>
-  <si>
-    <t>ST PIERRE ZERO LATA GREEN APPLE 24X310ML</t>
-  </si>
-  <si>
-    <t>CHICLETE TRIDENT MELANCIA C/21 UN</t>
-  </si>
-  <si>
-    <t>VINHO GRAVEDAD CARMENERE 750ML</t>
-  </si>
-  <si>
-    <t>NG AMOR CARIOCA BOMBOM BRANCO 500G</t>
-  </si>
-  <si>
-    <t>NG AMOR CARIOCA 200GR DUO (DP10 X20G)</t>
-  </si>
-  <si>
-    <t>WHISKY JIM BEAM RYE 700ML</t>
-  </si>
-  <si>
-    <t>CHICLETE TRIDENT MELANCIA C/ 14 UND</t>
-  </si>
-  <si>
-    <t>BOM AR AERO 360 ML CHEIRO DE TALCO</t>
-  </si>
-  <si>
-    <t>INSETICIDA SBP 360 ML ULTRA BARREIRA</t>
-  </si>
-  <si>
-    <t>4 PACK RED BULL SF BLUEBERRY BAUNILHA</t>
-  </si>
-  <si>
-    <t>4 PACK RED BULL SF NECTARINA 4X250ML</t>
-  </si>
-  <si>
-    <t>APERITIVO APEROL 750 ML</t>
-  </si>
-  <si>
-    <t>XAROPE MONIN MACA VERDE (APPLE) 700 ML</t>
-  </si>
-  <si>
-    <t>RED BULL SF NECTARINA 24X250ML</t>
-  </si>
-  <si>
-    <t>WHISKY J WALKER GREEN LABEL - 750ML</t>
-  </si>
-  <si>
-    <t>AGUA MINERAL MAMBA WATER C/ GAS 12X350ML</t>
-  </si>
-  <si>
-    <t>RED BULL CEREJA 24X250ML</t>
-  </si>
-  <si>
-    <t>AGUA NA LATA C/ GAS 12X310ML</t>
-  </si>
-  <si>
-    <t>XAROPE CHERRY MARIE BRIZARD 700ML</t>
-  </si>
-  <si>
-    <t>AGUA MINERAL MINALBA S/GAS LATA 12X310ML</t>
-  </si>
-  <si>
-    <t>VINHO ARESTI RESERVA CARMENERE 750ML</t>
-  </si>
-  <si>
-    <t>CERVEJA HEINEKEN ZERO LONG  24X330ML</t>
-  </si>
-  <si>
-    <t>VINHO HORIZONTE TINTO 750ML</t>
-  </si>
-  <si>
-    <t>LICOR CAN FIREBALL 750ML</t>
-  </si>
-  <si>
-    <t>FRISANTE MACAW TROPICAL MOSC. ROSE 750ML</t>
-  </si>
-  <si>
-    <t>FRISANTE MACAW TROPICAL MOSCATO 750ML</t>
-  </si>
-  <si>
-    <t>AGUA MINERAL MAMBA WATER S/ GAS 12X350ML</t>
-  </si>
-  <si>
-    <t>GIN INVICTUS MELANCIA 900ML</t>
-  </si>
-  <si>
-    <t>ESPUMANTE ARESTI CHARDONNAY 187,5ML</t>
-  </si>
-  <si>
-    <t>VINHO ARESTI ESTATE S. CARMENERE 750ML</t>
-  </si>
-  <si>
-    <t>TEQUILA EL JIMADOR REPOSADO 750 ML</t>
-  </si>
-  <si>
-    <t>NOSSO CHOP RED DRAFT VD 6X600ML</t>
-  </si>
-  <si>
-    <t>DRYCAT LONDON DRY GIN</t>
-  </si>
-  <si>
-    <t>GIN GORDONS PINK 700ML</t>
-  </si>
-  <si>
-    <t>VINHO ARESTI ESTATE S. CHARDONNAY 187ML</t>
-  </si>
-  <si>
-    <t>VINHO CAVAS DE ORO MALBEC 750ML</t>
-  </si>
-  <si>
-    <t>LICOR BANANINHA CARIOCA 750ML</t>
-  </si>
-  <si>
     <t>WHISKY J WALKER BLUE LABEL 750 ML</t>
   </si>
   <si>
@@ -23144,9 +23147,6 @@
   </si>
   <si>
     <t>XAROPE 1883 DE LIMAO SICILIANO 1L</t>
-  </si>
-  <si>
-    <t>VINHO TINTO BURDIZZO APPASSIMENTO 750ML</t>
   </si>
   <si>
     <t>4 PACK  RED BULL PITAYA</t>
@@ -35848,7 +35848,7 @@
         <v>6158</v>
       </c>
       <c r="D471" t="s">
-        <v>7402</v>
+        <v>7403</v>
       </c>
       <c r="E471" t="s">
         <v>7949</v>
@@ -49115,7 +49115,7 @@
         <v>6512</v>
       </c>
       <c r="D1100" t="s">
-        <v>7407</v>
+        <v>7561</v>
       </c>
       <c r="E1100" t="s">
         <v>7975</v>
@@ -49161,7 +49161,7 @@
         <v>6482</v>
       </c>
       <c r="D1102" t="s">
-        <v>7561</v>
+        <v>7562</v>
       </c>
       <c r="E1102" t="s">
         <v>7975</v>
@@ -49207,7 +49207,7 @@
         <v>6489</v>
       </c>
       <c r="D1104" t="s">
-        <v>7562</v>
+        <v>7563</v>
       </c>
       <c r="E1104" t="s">
         <v>7975</v>
@@ -49230,7 +49230,7 @@
         <v>6514</v>
       </c>
       <c r="D1105" t="s">
-        <v>7563</v>
+        <v>7564</v>
       </c>
       <c r="E1105" t="s">
         <v>7975</v>
@@ -49322,7 +49322,7 @@
         <v>6515</v>
       </c>
       <c r="D1109" t="s">
-        <v>7564</v>
+        <v>7565</v>
       </c>
       <c r="E1109" t="s">
         <v>7975</v>
@@ -49437,7 +49437,7 @@
         <v>6504</v>
       </c>
       <c r="D1114" t="s">
-        <v>7565</v>
+        <v>7566</v>
       </c>
       <c r="E1114" t="s">
         <v>7975</v>
@@ -49736,7 +49736,7 @@
         <v>6161</v>
       </c>
       <c r="D1127" t="s">
-        <v>7566</v>
+        <v>7567</v>
       </c>
       <c r="E1127" t="s">
         <v>7978</v>
@@ -49759,7 +49759,7 @@
         <v>6161</v>
       </c>
       <c r="D1128" t="s">
-        <v>7567</v>
+        <v>7568</v>
       </c>
       <c r="E1128" t="s">
         <v>7978</v>
@@ -49782,7 +49782,7 @@
         <v>6161</v>
       </c>
       <c r="D1129" t="s">
-        <v>7568</v>
+        <v>7569</v>
       </c>
       <c r="E1129" t="s">
         <v>7978</v>
@@ -49805,7 +49805,7 @@
         <v>5928</v>
       </c>
       <c r="D1130" t="s">
-        <v>7569</v>
+        <v>7570</v>
       </c>
       <c r="E1130" t="s">
         <v>7978</v>
@@ -49828,7 +49828,7 @@
         <v>6161</v>
       </c>
       <c r="D1131" t="s">
-        <v>7570</v>
+        <v>7571</v>
       </c>
       <c r="E1131" t="s">
         <v>7978</v>
@@ -49851,7 +49851,7 @@
         <v>6161</v>
       </c>
       <c r="D1132" t="s">
-        <v>7571</v>
+        <v>7572</v>
       </c>
       <c r="E1132" t="s">
         <v>7978</v>
@@ -49874,7 +49874,7 @@
         <v>6161</v>
       </c>
       <c r="D1133" t="s">
-        <v>7572</v>
+        <v>7573</v>
       </c>
       <c r="E1133" t="s">
         <v>7978</v>
@@ -49897,7 +49897,7 @@
         <v>5928</v>
       </c>
       <c r="D1134" t="s">
-        <v>7573</v>
+        <v>7574</v>
       </c>
       <c r="E1134" t="s">
         <v>7978</v>
@@ -49920,7 +49920,7 @@
         <v>6161</v>
       </c>
       <c r="D1135" t="s">
-        <v>7574</v>
+        <v>7575</v>
       </c>
       <c r="E1135" t="s">
         <v>7978</v>
@@ -49966,7 +49966,7 @@
         <v>5938</v>
       </c>
       <c r="D1137" t="s">
-        <v>7575</v>
+        <v>7576</v>
       </c>
       <c r="E1137" t="s">
         <v>7978</v>
@@ -49989,7 +49989,7 @@
         <v>5928</v>
       </c>
       <c r="D1138" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E1138" t="s">
         <v>7978</v>
@@ -50012,7 +50012,7 @@
         <v>6161</v>
       </c>
       <c r="D1139" t="s">
-        <v>7577</v>
+        <v>7578</v>
       </c>
       <c r="E1139" t="s">
         <v>7978</v>
@@ -50035,7 +50035,7 @@
         <v>6161</v>
       </c>
       <c r="D1140" t="s">
-        <v>7568</v>
+        <v>7569</v>
       </c>
       <c r="E1140" t="s">
         <v>7978</v>
@@ -50058,7 +50058,7 @@
         <v>5928</v>
       </c>
       <c r="D1141" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1141" t="s">
         <v>7978</v>
@@ -50081,7 +50081,7 @@
         <v>6161</v>
       </c>
       <c r="D1142" t="s">
-        <v>7574</v>
+        <v>7575</v>
       </c>
       <c r="E1142" t="s">
         <v>7978</v>
@@ -50104,7 +50104,7 @@
         <v>5928</v>
       </c>
       <c r="D1143" t="s">
-        <v>7572</v>
+        <v>7573</v>
       </c>
       <c r="E1143" t="s">
         <v>7978</v>
@@ -50127,7 +50127,7 @@
         <v>5928</v>
       </c>
       <c r="D1144" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1144" t="s">
         <v>7978</v>
@@ -50150,7 +50150,7 @@
         <v>5928</v>
       </c>
       <c r="D1145" t="s">
-        <v>7577</v>
+        <v>7578</v>
       </c>
       <c r="E1145" t="s">
         <v>7978</v>
@@ -50173,7 +50173,7 @@
         <v>6161</v>
       </c>
       <c r="D1146" t="s">
-        <v>7579</v>
+        <v>7580</v>
       </c>
       <c r="E1146" t="s">
         <v>7978</v>
@@ -50196,7 +50196,7 @@
         <v>6161</v>
       </c>
       <c r="D1147" t="s">
-        <v>7580</v>
+        <v>7581</v>
       </c>
       <c r="E1147" t="s">
         <v>7978</v>
@@ -50219,7 +50219,7 @@
         <v>6522</v>
       </c>
       <c r="D1148" t="s">
-        <v>7581</v>
+        <v>7582</v>
       </c>
       <c r="E1148" t="s">
         <v>7978</v>
@@ -50265,7 +50265,7 @@
         <v>5938</v>
       </c>
       <c r="D1150" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1150" t="s">
         <v>7978</v>
@@ -50288,7 +50288,7 @@
         <v>6161</v>
       </c>
       <c r="D1151" t="s">
-        <v>7583</v>
+        <v>7584</v>
       </c>
       <c r="E1151" t="s">
         <v>7978</v>
@@ -50311,7 +50311,7 @@
         <v>6161</v>
       </c>
       <c r="D1152" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1152" t="s">
         <v>7978</v>
@@ -50334,7 +50334,7 @@
         <v>6523</v>
       </c>
       <c r="D1153" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1153" t="s">
         <v>7978</v>
@@ -50357,7 +50357,7 @@
         <v>6161</v>
       </c>
       <c r="D1154" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1154" t="s">
         <v>7978</v>
@@ -50403,7 +50403,7 @@
         <v>5928</v>
       </c>
       <c r="D1156" t="s">
-        <v>7586</v>
+        <v>7587</v>
       </c>
       <c r="E1156" t="s">
         <v>7978</v>
@@ -50426,7 +50426,7 @@
         <v>6161</v>
       </c>
       <c r="D1157" t="s">
-        <v>7586</v>
+        <v>7587</v>
       </c>
       <c r="E1157" t="s">
         <v>7978</v>
@@ -50472,7 +50472,7 @@
         <v>6161</v>
       </c>
       <c r="D1159" t="s">
-        <v>7587</v>
+        <v>7588</v>
       </c>
       <c r="E1159" t="s">
         <v>7978</v>
@@ -50495,7 +50495,7 @@
         <v>6161</v>
       </c>
       <c r="D1160" t="s">
-        <v>7587</v>
+        <v>7588</v>
       </c>
       <c r="E1160" t="s">
         <v>7978</v>
@@ -50518,7 +50518,7 @@
         <v>6161</v>
       </c>
       <c r="D1161" t="s">
-        <v>7580</v>
+        <v>7581</v>
       </c>
       <c r="E1161" t="s">
         <v>7978</v>
@@ -50541,7 +50541,7 @@
         <v>6161</v>
       </c>
       <c r="D1162" t="s">
-        <v>7586</v>
+        <v>7587</v>
       </c>
       <c r="E1162" t="s">
         <v>7978</v>
@@ -50610,7 +50610,7 @@
         <v>6161</v>
       </c>
       <c r="D1165" t="s">
-        <v>7588</v>
+        <v>7589</v>
       </c>
       <c r="E1165" t="s">
         <v>7978</v>
@@ -50633,7 +50633,7 @@
         <v>6161</v>
       </c>
       <c r="D1166" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1166" t="s">
         <v>7978</v>
@@ -50656,7 +50656,7 @@
         <v>5938</v>
       </c>
       <c r="D1167" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1167" t="s">
         <v>7978</v>
@@ -50679,7 +50679,7 @@
         <v>6161</v>
       </c>
       <c r="D1168" t="s">
-        <v>7589</v>
+        <v>7590</v>
       </c>
       <c r="E1168" t="s">
         <v>7978</v>
@@ -50725,7 +50725,7 @@
         <v>6161</v>
       </c>
       <c r="D1170" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E1170" t="s">
         <v>7978</v>
@@ -50794,7 +50794,7 @@
         <v>6526</v>
       </c>
       <c r="D1173" t="s">
-        <v>7574</v>
+        <v>7575</v>
       </c>
       <c r="E1173" t="s">
         <v>7978</v>
@@ -50840,7 +50840,7 @@
         <v>6161</v>
       </c>
       <c r="D1175" t="s">
-        <v>7590</v>
+        <v>7591</v>
       </c>
       <c r="E1175" t="s">
         <v>7978</v>
@@ -50863,7 +50863,7 @@
         <v>6161</v>
       </c>
       <c r="D1176" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1176" t="s">
         <v>7978</v>
@@ -50886,7 +50886,7 @@
         <v>6161</v>
       </c>
       <c r="D1177" t="s">
-        <v>7587</v>
+        <v>7588</v>
       </c>
       <c r="E1177" t="s">
         <v>7978</v>
@@ -50932,7 +50932,7 @@
         <v>6161</v>
       </c>
       <c r="D1179" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1179" t="s">
         <v>7978</v>
@@ -50955,7 +50955,7 @@
         <v>6161</v>
       </c>
       <c r="D1180" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1180" t="s">
         <v>7978</v>
@@ -50978,7 +50978,7 @@
         <v>6161</v>
       </c>
       <c r="D1181" t="s">
-        <v>7591</v>
+        <v>7592</v>
       </c>
       <c r="E1181" t="s">
         <v>7978</v>
@@ -51024,7 +51024,7 @@
         <v>5938</v>
       </c>
       <c r="D1183" t="s">
-        <v>7579</v>
+        <v>7580</v>
       </c>
       <c r="E1183" t="s">
         <v>7978</v>
@@ -51047,7 +51047,7 @@
         <v>6161</v>
       </c>
       <c r="D1184" t="s">
-        <v>7589</v>
+        <v>7590</v>
       </c>
       <c r="E1184" t="s">
         <v>7978</v>
@@ -51093,7 +51093,7 @@
         <v>5928</v>
       </c>
       <c r="D1186" t="s">
-        <v>7592</v>
+        <v>7593</v>
       </c>
       <c r="E1186" t="s">
         <v>7978</v>
@@ -51116,7 +51116,7 @@
         <v>5928</v>
       </c>
       <c r="D1187" t="s">
-        <v>7593</v>
+        <v>7594</v>
       </c>
       <c r="E1187" t="s">
         <v>7978</v>
@@ -51185,7 +51185,7 @@
         <v>6161</v>
       </c>
       <c r="D1190" t="s">
-        <v>7594</v>
+        <v>7595</v>
       </c>
       <c r="E1190" t="s">
         <v>7978</v>
@@ -51208,7 +51208,7 @@
         <v>5938</v>
       </c>
       <c r="D1191" t="s">
-        <v>7595</v>
+        <v>7596</v>
       </c>
       <c r="E1191" t="s">
         <v>7978</v>
@@ -51231,7 +51231,7 @@
         <v>5938</v>
       </c>
       <c r="D1192" t="s">
-        <v>7596</v>
+        <v>7597</v>
       </c>
       <c r="E1192" t="s">
         <v>7978</v>
@@ -51254,7 +51254,7 @@
         <v>6161</v>
       </c>
       <c r="D1193" t="s">
-        <v>7597</v>
+        <v>7598</v>
       </c>
       <c r="E1193" t="s">
         <v>7978</v>
@@ -51277,7 +51277,7 @@
         <v>6528</v>
       </c>
       <c r="D1194" t="s">
-        <v>7598</v>
+        <v>7599</v>
       </c>
       <c r="E1194" t="s">
         <v>7978</v>
@@ -51300,7 +51300,7 @@
         <v>5909</v>
       </c>
       <c r="D1195" t="s">
-        <v>7595</v>
+        <v>7596</v>
       </c>
       <c r="E1195" t="s">
         <v>7978</v>
@@ -51346,7 +51346,7 @@
         <v>6161</v>
       </c>
       <c r="D1197" t="s">
-        <v>7599</v>
+        <v>7600</v>
       </c>
       <c r="E1197" t="s">
         <v>7978</v>
@@ -51369,7 +51369,7 @@
         <v>6161</v>
       </c>
       <c r="D1198" t="s">
-        <v>7600</v>
+        <v>7601</v>
       </c>
       <c r="E1198" t="s">
         <v>7978</v>
@@ -51415,7 +51415,7 @@
         <v>6161</v>
       </c>
       <c r="D1200" t="s">
-        <v>7601</v>
+        <v>7602</v>
       </c>
       <c r="E1200" t="s">
         <v>7978</v>
@@ -51438,7 +51438,7 @@
         <v>6161</v>
       </c>
       <c r="D1201" t="s">
-        <v>7601</v>
+        <v>7602</v>
       </c>
       <c r="E1201" t="s">
         <v>7978</v>
@@ -51461,7 +51461,7 @@
         <v>5928</v>
       </c>
       <c r="D1202" t="s">
-        <v>7602</v>
+        <v>7603</v>
       </c>
       <c r="E1202" t="s">
         <v>7978</v>
@@ -51484,7 +51484,7 @@
         <v>6161</v>
       </c>
       <c r="D1203" t="s">
-        <v>7603</v>
+        <v>7604</v>
       </c>
       <c r="E1203" t="s">
         <v>7978</v>
@@ -51507,7 +51507,7 @@
         <v>6161</v>
       </c>
       <c r="D1204" t="s">
-        <v>7604</v>
+        <v>7605</v>
       </c>
       <c r="E1204" t="s">
         <v>7978</v>
@@ -51530,7 +51530,7 @@
         <v>5928</v>
       </c>
       <c r="D1205" t="s">
-        <v>7603</v>
+        <v>7604</v>
       </c>
       <c r="E1205" t="s">
         <v>7978</v>
@@ -51576,7 +51576,7 @@
         <v>6161</v>
       </c>
       <c r="D1207" t="s">
-        <v>7605</v>
+        <v>7606</v>
       </c>
       <c r="E1207" t="s">
         <v>7978</v>
@@ -51599,7 +51599,7 @@
         <v>5938</v>
       </c>
       <c r="D1208" t="s">
-        <v>7606</v>
+        <v>7607</v>
       </c>
       <c r="E1208" t="s">
         <v>7978</v>
@@ -51622,7 +51622,7 @@
         <v>5938</v>
       </c>
       <c r="D1209" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1209" t="s">
         <v>7978</v>
@@ -51691,7 +51691,7 @@
         <v>5928</v>
       </c>
       <c r="D1212" t="s">
-        <v>7607</v>
+        <v>7608</v>
       </c>
       <c r="E1212" t="s">
         <v>7978</v>
@@ -51714,7 +51714,7 @@
         <v>6161</v>
       </c>
       <c r="D1213" t="s">
-        <v>7608</v>
+        <v>7609</v>
       </c>
       <c r="E1213" t="s">
         <v>7978</v>
@@ -51737,7 +51737,7 @@
         <v>5938</v>
       </c>
       <c r="D1214" t="s">
-        <v>7609</v>
+        <v>7610</v>
       </c>
       <c r="E1214" t="s">
         <v>7978</v>
@@ -51760,7 +51760,7 @@
         <v>6529</v>
       </c>
       <c r="D1215" t="s">
-        <v>7610</v>
+        <v>7611</v>
       </c>
       <c r="E1215" t="s">
         <v>7978</v>
@@ -51783,7 +51783,7 @@
         <v>6529</v>
       </c>
       <c r="D1216" t="s">
-        <v>7610</v>
+        <v>7611</v>
       </c>
       <c r="E1216" t="s">
         <v>7978</v>
@@ -51806,7 +51806,7 @@
         <v>6161</v>
       </c>
       <c r="D1217" t="s">
-        <v>7611</v>
+        <v>7612</v>
       </c>
       <c r="E1217" t="s">
         <v>7978</v>
@@ -51875,7 +51875,7 @@
         <v>6161</v>
       </c>
       <c r="D1220" t="s">
-        <v>7612</v>
+        <v>7613</v>
       </c>
       <c r="E1220" t="s">
         <v>7978</v>
@@ -51967,7 +51967,7 @@
         <v>6161</v>
       </c>
       <c r="D1224" t="s">
-        <v>7594</v>
+        <v>7595</v>
       </c>
       <c r="E1224" t="s">
         <v>7978</v>
@@ -51990,7 +51990,7 @@
         <v>6161</v>
       </c>
       <c r="D1225" t="s">
-        <v>7613</v>
+        <v>7614</v>
       </c>
       <c r="E1225" t="s">
         <v>7978</v>
@@ -52059,7 +52059,7 @@
         <v>5928</v>
       </c>
       <c r="D1228" t="s">
-        <v>7596</v>
+        <v>7597</v>
       </c>
       <c r="E1228" t="s">
         <v>7978</v>
@@ -52082,7 +52082,7 @@
         <v>5928</v>
       </c>
       <c r="D1229" t="s">
-        <v>7614</v>
+        <v>7615</v>
       </c>
       <c r="E1229" t="s">
         <v>7978</v>
@@ -52128,7 +52128,7 @@
         <v>6161</v>
       </c>
       <c r="D1231" t="s">
-        <v>7615</v>
+        <v>7616</v>
       </c>
       <c r="E1231" t="s">
         <v>7978</v>
@@ -52151,7 +52151,7 @@
         <v>6161</v>
       </c>
       <c r="D1232" t="s">
-        <v>7577</v>
+        <v>7578</v>
       </c>
       <c r="E1232" t="s">
         <v>7978</v>
@@ -52174,7 +52174,7 @@
         <v>5938</v>
       </c>
       <c r="D1233" t="s">
-        <v>7616</v>
+        <v>7617</v>
       </c>
       <c r="E1233" t="s">
         <v>7978</v>
@@ -52197,7 +52197,7 @@
         <v>6161</v>
       </c>
       <c r="D1234" t="s">
-        <v>7617</v>
+        <v>7618</v>
       </c>
       <c r="E1234" t="s">
         <v>7978</v>
@@ -52220,7 +52220,7 @@
         <v>6161</v>
       </c>
       <c r="D1235" t="s">
-        <v>7617</v>
+        <v>7618</v>
       </c>
       <c r="E1235" t="s">
         <v>7978</v>
@@ -52243,7 +52243,7 @@
         <v>6161</v>
       </c>
       <c r="D1236" t="s">
-        <v>7618</v>
+        <v>7619</v>
       </c>
       <c r="E1236" t="s">
         <v>7978</v>
@@ -52266,7 +52266,7 @@
         <v>5928</v>
       </c>
       <c r="D1237" t="s">
-        <v>7619</v>
+        <v>7620</v>
       </c>
       <c r="E1237" t="s">
         <v>7978</v>
@@ -52312,7 +52312,7 @@
         <v>6161</v>
       </c>
       <c r="D1239" t="s">
-        <v>7599</v>
+        <v>7600</v>
       </c>
       <c r="E1239" t="s">
         <v>7978</v>
@@ -52335,7 +52335,7 @@
         <v>6161</v>
       </c>
       <c r="D1240" t="s">
-        <v>7568</v>
+        <v>7569</v>
       </c>
       <c r="E1240" t="s">
         <v>7978</v>
@@ -52358,7 +52358,7 @@
         <v>5928</v>
       </c>
       <c r="D1241" t="s">
-        <v>7620</v>
+        <v>7621</v>
       </c>
       <c r="E1241" t="s">
         <v>7978</v>
@@ -52381,7 +52381,7 @@
         <v>6161</v>
       </c>
       <c r="D1242" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1242" t="s">
         <v>7978</v>
@@ -52404,7 +52404,7 @@
         <v>5928</v>
       </c>
       <c r="D1243" t="s">
-        <v>7620</v>
+        <v>7621</v>
       </c>
       <c r="E1243" t="s">
         <v>7978</v>
@@ -52427,7 +52427,7 @@
         <v>6161</v>
       </c>
       <c r="D1244" t="s">
-        <v>7621</v>
+        <v>7622</v>
       </c>
       <c r="E1244" t="s">
         <v>7978</v>
@@ -52450,7 +52450,7 @@
         <v>5938</v>
       </c>
       <c r="D1245" t="s">
-        <v>7622</v>
+        <v>7623</v>
       </c>
       <c r="E1245" t="s">
         <v>7978</v>
@@ -52473,7 +52473,7 @@
         <v>5938</v>
       </c>
       <c r="D1246" t="s">
-        <v>7623</v>
+        <v>7624</v>
       </c>
       <c r="E1246" t="s">
         <v>7978</v>
@@ -52496,7 +52496,7 @@
         <v>6161</v>
       </c>
       <c r="D1247" t="s">
-        <v>7572</v>
+        <v>7573</v>
       </c>
       <c r="E1247" t="s">
         <v>7978</v>
@@ -52519,7 +52519,7 @@
         <v>5928</v>
       </c>
       <c r="D1248" t="s">
-        <v>7624</v>
+        <v>7625</v>
       </c>
       <c r="E1248" t="s">
         <v>7978</v>
@@ -52565,7 +52565,7 @@
         <v>6161</v>
       </c>
       <c r="D1250" t="s">
-        <v>7625</v>
+        <v>7626</v>
       </c>
       <c r="E1250" t="s">
         <v>7978</v>
@@ -52588,7 +52588,7 @@
         <v>5928</v>
       </c>
       <c r="D1251" t="s">
-        <v>7626</v>
+        <v>7627</v>
       </c>
       <c r="E1251" t="s">
         <v>7978</v>
@@ -52634,7 +52634,7 @@
         <v>6161</v>
       </c>
       <c r="D1253" t="s">
-        <v>7627</v>
+        <v>7628</v>
       </c>
       <c r="E1253" t="s">
         <v>7978</v>
@@ -52726,7 +52726,7 @@
         <v>5938</v>
       </c>
       <c r="D1257" t="s">
-        <v>7628</v>
+        <v>7629</v>
       </c>
       <c r="E1257" t="s">
         <v>7978</v>
@@ -52749,7 +52749,7 @@
         <v>6161</v>
       </c>
       <c r="D1258" t="s">
-        <v>7629</v>
+        <v>7630</v>
       </c>
       <c r="E1258" t="s">
         <v>7978</v>
@@ -52772,7 +52772,7 @@
         <v>6161</v>
       </c>
       <c r="D1259" t="s">
-        <v>7630</v>
+        <v>7631</v>
       </c>
       <c r="E1259" t="s">
         <v>7978</v>
@@ -52795,7 +52795,7 @@
         <v>5928</v>
       </c>
       <c r="D1260" t="s">
-        <v>7631</v>
+        <v>7632</v>
       </c>
       <c r="E1260" t="s">
         <v>7978</v>
@@ -52841,7 +52841,7 @@
         <v>6161</v>
       </c>
       <c r="D1262" t="s">
-        <v>7632</v>
+        <v>7633</v>
       </c>
       <c r="E1262" t="s">
         <v>7978</v>
@@ -52910,7 +52910,7 @@
         <v>6161</v>
       </c>
       <c r="D1265" t="s">
-        <v>7633</v>
+        <v>7634</v>
       </c>
       <c r="E1265" t="s">
         <v>7978</v>
@@ -52979,7 +52979,7 @@
         <v>5928</v>
       </c>
       <c r="D1268" t="s">
-        <v>7575</v>
+        <v>7576</v>
       </c>
       <c r="E1268" t="s">
         <v>7978</v>
@@ -53002,7 +53002,7 @@
         <v>5928</v>
       </c>
       <c r="D1269" t="s">
-        <v>7634</v>
+        <v>7635</v>
       </c>
       <c r="E1269" t="s">
         <v>7978</v>
@@ -53025,7 +53025,7 @@
         <v>5928</v>
       </c>
       <c r="D1270" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1270" t="s">
         <v>7978</v>
@@ -53071,7 +53071,7 @@
         <v>6161</v>
       </c>
       <c r="D1272" t="s">
-        <v>7635</v>
+        <v>7636</v>
       </c>
       <c r="E1272" t="s">
         <v>7978</v>
@@ -53094,7 +53094,7 @@
         <v>5928</v>
       </c>
       <c r="D1273" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E1273" t="s">
         <v>7978</v>
@@ -53117,7 +53117,7 @@
         <v>6161</v>
       </c>
       <c r="D1274" t="s">
-        <v>7636</v>
+        <v>7637</v>
       </c>
       <c r="E1274" t="s">
         <v>7978</v>
@@ -53140,7 +53140,7 @@
         <v>6161</v>
       </c>
       <c r="D1275" t="s">
-        <v>7637</v>
+        <v>7638</v>
       </c>
       <c r="E1275" t="s">
         <v>7978</v>
@@ -53186,7 +53186,7 @@
         <v>6161</v>
       </c>
       <c r="D1277" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1277" t="s">
         <v>7978</v>
@@ -53209,7 +53209,7 @@
         <v>5938</v>
       </c>
       <c r="D1278" t="s">
-        <v>7619</v>
+        <v>7620</v>
       </c>
       <c r="E1278" t="s">
         <v>7978</v>
@@ -53301,7 +53301,7 @@
         <v>6161</v>
       </c>
       <c r="D1282" t="s">
-        <v>7638</v>
+        <v>7639</v>
       </c>
       <c r="E1282" t="s">
         <v>7978</v>
@@ -53324,7 +53324,7 @@
         <v>6161</v>
       </c>
       <c r="D1283" t="s">
-        <v>7568</v>
+        <v>7569</v>
       </c>
       <c r="E1283" t="s">
         <v>7978</v>
@@ -53370,7 +53370,7 @@
         <v>5938</v>
       </c>
       <c r="D1285" t="s">
-        <v>7639</v>
+        <v>7640</v>
       </c>
       <c r="E1285" t="s">
         <v>7978</v>
@@ -53393,7 +53393,7 @@
         <v>5928</v>
       </c>
       <c r="D1286" t="s">
-        <v>7640</v>
+        <v>7641</v>
       </c>
       <c r="E1286" t="s">
         <v>7978</v>
@@ -53439,7 +53439,7 @@
         <v>5928</v>
       </c>
       <c r="D1288" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1288" t="s">
         <v>7978</v>
@@ -53485,7 +53485,7 @@
         <v>6161</v>
       </c>
       <c r="D1290" t="s">
-        <v>7567</v>
+        <v>7568</v>
       </c>
       <c r="E1290" t="s">
         <v>7978</v>
@@ -53508,7 +53508,7 @@
         <v>6016</v>
       </c>
       <c r="D1291" t="s">
-        <v>7641</v>
+        <v>7642</v>
       </c>
       <c r="E1291" t="s">
         <v>7978</v>
@@ -53531,7 +53531,7 @@
         <v>6161</v>
       </c>
       <c r="D1292" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1292" t="s">
         <v>7978</v>
@@ -53577,7 +53577,7 @@
         <v>6161</v>
       </c>
       <c r="D1294" t="s">
-        <v>7574</v>
+        <v>7575</v>
       </c>
       <c r="E1294" t="s">
         <v>7978</v>
@@ -53600,7 +53600,7 @@
         <v>5938</v>
       </c>
       <c r="D1295" t="s">
-        <v>7642</v>
+        <v>7643</v>
       </c>
       <c r="E1295" t="s">
         <v>7978</v>
@@ -53623,7 +53623,7 @@
         <v>6161</v>
       </c>
       <c r="D1296" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1296" t="s">
         <v>7978</v>
@@ -53715,7 +53715,7 @@
         <v>6161</v>
       </c>
       <c r="D1300" t="s">
-        <v>7643</v>
+        <v>7644</v>
       </c>
       <c r="E1300" t="s">
         <v>7978</v>
@@ -53738,7 +53738,7 @@
         <v>6161</v>
       </c>
       <c r="D1301" t="s">
-        <v>7644</v>
+        <v>7645</v>
       </c>
       <c r="E1301" t="s">
         <v>7978</v>
@@ -53761,7 +53761,7 @@
         <v>6161</v>
       </c>
       <c r="D1302" t="s">
-        <v>7624</v>
+        <v>7625</v>
       </c>
       <c r="E1302" t="s">
         <v>7978</v>
@@ -53784,7 +53784,7 @@
         <v>5928</v>
       </c>
       <c r="D1303" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1303" t="s">
         <v>7978</v>
@@ -53830,7 +53830,7 @@
         <v>6161</v>
       </c>
       <c r="D1305" t="s">
-        <v>7572</v>
+        <v>7573</v>
       </c>
       <c r="E1305" t="s">
         <v>7978</v>
@@ -53853,7 +53853,7 @@
         <v>5928</v>
       </c>
       <c r="D1306" t="s">
-        <v>7645</v>
+        <v>7646</v>
       </c>
       <c r="E1306" t="s">
         <v>7978</v>
@@ -53899,7 +53899,7 @@
         <v>5938</v>
       </c>
       <c r="D1308" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1308" t="s">
         <v>7978</v>
@@ -53922,7 +53922,7 @@
         <v>6015</v>
       </c>
       <c r="D1309" t="s">
-        <v>7646</v>
+        <v>7647</v>
       </c>
       <c r="E1309" t="s">
         <v>7978</v>
@@ -53945,7 +53945,7 @@
         <v>6161</v>
       </c>
       <c r="D1310" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1310" t="s">
         <v>7978</v>
@@ -53991,7 +53991,7 @@
         <v>6161</v>
       </c>
       <c r="D1312" t="s">
-        <v>7587</v>
+        <v>7588</v>
       </c>
       <c r="E1312" t="s">
         <v>7978</v>
@@ -54014,7 +54014,7 @@
         <v>5952</v>
       </c>
       <c r="D1313" t="s">
-        <v>7647</v>
+        <v>7648</v>
       </c>
       <c r="E1313" t="s">
         <v>7978</v>
@@ -54037,7 +54037,7 @@
         <v>6161</v>
       </c>
       <c r="D1314" t="s">
-        <v>7648</v>
+        <v>7649</v>
       </c>
       <c r="E1314" t="s">
         <v>7978</v>
@@ -54083,7 +54083,7 @@
         <v>6161</v>
       </c>
       <c r="D1316" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1316" t="s">
         <v>7978</v>
@@ -54129,7 +54129,7 @@
         <v>5928</v>
       </c>
       <c r="D1318" t="s">
-        <v>7649</v>
+        <v>7650</v>
       </c>
       <c r="E1318" t="s">
         <v>7978</v>
@@ -54152,7 +54152,7 @@
         <v>6530</v>
       </c>
       <c r="D1319" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1319" t="s">
         <v>7978</v>
@@ -54175,7 +54175,7 @@
         <v>5938</v>
       </c>
       <c r="D1320" t="s">
-        <v>7650</v>
+        <v>7651</v>
       </c>
       <c r="E1320" t="s">
         <v>7978</v>
@@ -54198,7 +54198,7 @@
         <v>6530</v>
       </c>
       <c r="D1321" t="s">
-        <v>7651</v>
+        <v>7652</v>
       </c>
       <c r="E1321" t="s">
         <v>7978</v>
@@ -54221,7 +54221,7 @@
         <v>5938</v>
       </c>
       <c r="D1322" t="s">
-        <v>7568</v>
+        <v>7569</v>
       </c>
       <c r="E1322" t="s">
         <v>7978</v>
@@ -54267,7 +54267,7 @@
         <v>5938</v>
       </c>
       <c r="D1324" t="s">
-        <v>7652</v>
+        <v>7653</v>
       </c>
       <c r="E1324" t="s">
         <v>7978</v>
@@ -54290,7 +54290,7 @@
         <v>5938</v>
       </c>
       <c r="D1325" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1325" t="s">
         <v>7978</v>
@@ -54313,7 +54313,7 @@
         <v>6013</v>
       </c>
       <c r="D1326" t="s">
-        <v>7653</v>
+        <v>7654</v>
       </c>
       <c r="E1326" t="s">
         <v>7978</v>
@@ -54336,7 +54336,7 @@
         <v>6161</v>
       </c>
       <c r="D1327" t="s">
-        <v>7568</v>
+        <v>7569</v>
       </c>
       <c r="E1327" t="s">
         <v>7978</v>
@@ -54359,7 +54359,7 @@
         <v>6161</v>
       </c>
       <c r="D1328" t="s">
-        <v>7568</v>
+        <v>7569</v>
       </c>
       <c r="E1328" t="s">
         <v>7978</v>
@@ -54382,7 +54382,7 @@
         <v>6161</v>
       </c>
       <c r="D1329" t="s">
-        <v>7571</v>
+        <v>7572</v>
       </c>
       <c r="E1329" t="s">
         <v>7978</v>
@@ -54428,7 +54428,7 @@
         <v>5938</v>
       </c>
       <c r="D1331" t="s">
-        <v>7654</v>
+        <v>7655</v>
       </c>
       <c r="E1331" t="s">
         <v>7978</v>
@@ -54474,7 +54474,7 @@
         <v>5938</v>
       </c>
       <c r="D1333" t="s">
-        <v>7655</v>
+        <v>7656</v>
       </c>
       <c r="E1333" t="s">
         <v>7978</v>
@@ -54497,7 +54497,7 @@
         <v>5928</v>
       </c>
       <c r="D1334" t="s">
-        <v>7570</v>
+        <v>7571</v>
       </c>
       <c r="E1334" t="s">
         <v>7978</v>
@@ -54543,7 +54543,7 @@
         <v>6161</v>
       </c>
       <c r="D1336" t="s">
-        <v>7656</v>
+        <v>7657</v>
       </c>
       <c r="E1336" t="s">
         <v>7978</v>
@@ -54566,7 +54566,7 @@
         <v>5938</v>
       </c>
       <c r="D1337" t="s">
-        <v>7568</v>
+        <v>7569</v>
       </c>
       <c r="E1337" t="s">
         <v>7978</v>
@@ -54589,7 +54589,7 @@
         <v>5928</v>
       </c>
       <c r="D1338" t="s">
-        <v>7657</v>
+        <v>7658</v>
       </c>
       <c r="E1338" t="s">
         <v>7978</v>
@@ -54612,7 +54612,7 @@
         <v>5928</v>
       </c>
       <c r="D1339" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1339" t="s">
         <v>7978</v>
@@ -54635,7 +54635,7 @@
         <v>6161</v>
       </c>
       <c r="D1340" t="s">
-        <v>7641</v>
+        <v>7642</v>
       </c>
       <c r="E1340" t="s">
         <v>7978</v>
@@ -54681,7 +54681,7 @@
         <v>6119</v>
       </c>
       <c r="D1342" t="s">
-        <v>7580</v>
+        <v>7581</v>
       </c>
       <c r="E1342" t="s">
         <v>7978</v>
@@ -54750,7 +54750,7 @@
         <v>5928</v>
       </c>
       <c r="D1345" t="s">
-        <v>7658</v>
+        <v>7659</v>
       </c>
       <c r="E1345" t="s">
         <v>7978</v>
@@ -54773,7 +54773,7 @@
         <v>6533</v>
       </c>
       <c r="D1346" t="s">
-        <v>7659</v>
+        <v>7660</v>
       </c>
       <c r="E1346" t="s">
         <v>7978</v>
@@ -54796,7 +54796,7 @@
         <v>6161</v>
       </c>
       <c r="D1347" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1347" t="s">
         <v>7978</v>
@@ -54842,7 +54842,7 @@
         <v>6161</v>
       </c>
       <c r="D1349" t="s">
-        <v>7660</v>
+        <v>7661</v>
       </c>
       <c r="E1349" t="s">
         <v>7978</v>
@@ -54865,7 +54865,7 @@
         <v>5934</v>
       </c>
       <c r="D1350" t="s">
-        <v>7661</v>
+        <v>7662</v>
       </c>
       <c r="E1350" t="s">
         <v>7978</v>
@@ -54911,7 +54911,7 @@
         <v>6534</v>
       </c>
       <c r="D1352" t="s">
-        <v>7662</v>
+        <v>7663</v>
       </c>
       <c r="E1352" t="s">
         <v>7978</v>
@@ -54957,7 +54957,7 @@
         <v>6161</v>
       </c>
       <c r="D1354" t="s">
-        <v>7644</v>
+        <v>7645</v>
       </c>
       <c r="E1354" t="s">
         <v>7978</v>
@@ -54980,7 +54980,7 @@
         <v>6161</v>
       </c>
       <c r="D1355" t="s">
-        <v>7567</v>
+        <v>7568</v>
       </c>
       <c r="E1355" t="s">
         <v>7978</v>
@@ -55003,7 +55003,7 @@
         <v>5928</v>
       </c>
       <c r="D1356" t="s">
-        <v>7572</v>
+        <v>7573</v>
       </c>
       <c r="E1356" t="s">
         <v>7978</v>
@@ -55026,7 +55026,7 @@
         <v>6161</v>
       </c>
       <c r="D1357" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1357" t="s">
         <v>7978</v>
@@ -55049,7 +55049,7 @@
         <v>6161</v>
       </c>
       <c r="D1358" t="s">
-        <v>7645</v>
+        <v>7646</v>
       </c>
       <c r="E1358" t="s">
         <v>7978</v>
@@ -55072,7 +55072,7 @@
         <v>6161</v>
       </c>
       <c r="D1359" t="s">
-        <v>7591</v>
+        <v>7592</v>
       </c>
       <c r="E1359" t="s">
         <v>7978</v>
@@ -55095,7 +55095,7 @@
         <v>6161</v>
       </c>
       <c r="D1360" t="s">
-        <v>7663</v>
+        <v>7664</v>
       </c>
       <c r="E1360" t="s">
         <v>7978</v>
@@ -55118,7 +55118,7 @@
         <v>6161</v>
       </c>
       <c r="D1361" t="s">
-        <v>7589</v>
+        <v>7590</v>
       </c>
       <c r="E1361" t="s">
         <v>7978</v>
@@ -55141,7 +55141,7 @@
         <v>5938</v>
       </c>
       <c r="D1362" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1362" t="s">
         <v>7978</v>
@@ -55164,7 +55164,7 @@
         <v>6161</v>
       </c>
       <c r="D1363" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1363" t="s">
         <v>7978</v>
@@ -55187,7 +55187,7 @@
         <v>6535</v>
       </c>
       <c r="D1364" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1364" t="s">
         <v>7978</v>
@@ -55210,7 +55210,7 @@
         <v>5930</v>
       </c>
       <c r="D1365" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1365" t="s">
         <v>7978</v>
@@ -55279,7 +55279,7 @@
         <v>5928</v>
       </c>
       <c r="D1368" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1368" t="s">
         <v>7978</v>
@@ -55302,7 +55302,7 @@
         <v>6161</v>
       </c>
       <c r="D1369" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1369" t="s">
         <v>7978</v>
@@ -55325,7 +55325,7 @@
         <v>6161</v>
       </c>
       <c r="D1370" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1370" t="s">
         <v>7978</v>
@@ -55348,7 +55348,7 @@
         <v>6161</v>
       </c>
       <c r="D1371" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1371" t="s">
         <v>7978</v>
@@ -55371,7 +55371,7 @@
         <v>6161</v>
       </c>
       <c r="D1372" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1372" t="s">
         <v>7978</v>
@@ -55417,7 +55417,7 @@
         <v>6161</v>
       </c>
       <c r="D1374" t="s">
-        <v>7664</v>
+        <v>7665</v>
       </c>
       <c r="E1374" t="s">
         <v>7978</v>
@@ -55440,7 +55440,7 @@
         <v>6161</v>
       </c>
       <c r="D1375" t="s">
-        <v>7596</v>
+        <v>7597</v>
       </c>
       <c r="E1375" t="s">
         <v>7978</v>
@@ -55486,7 +55486,7 @@
         <v>5928</v>
       </c>
       <c r="D1377" t="s">
-        <v>7665</v>
+        <v>7666</v>
       </c>
       <c r="E1377" t="s">
         <v>7978</v>
@@ -55509,7 +55509,7 @@
         <v>6161</v>
       </c>
       <c r="D1378" t="s">
-        <v>7624</v>
+        <v>7625</v>
       </c>
       <c r="E1378" t="s">
         <v>7978</v>
@@ -55532,7 +55532,7 @@
         <v>5928</v>
       </c>
       <c r="D1379" t="s">
-        <v>7666</v>
+        <v>7667</v>
       </c>
       <c r="E1379" t="s">
         <v>7978</v>
@@ -55624,7 +55624,7 @@
         <v>5938</v>
       </c>
       <c r="D1383" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1383" t="s">
         <v>7978</v>
@@ -55647,7 +55647,7 @@
         <v>5913</v>
       </c>
       <c r="D1384" t="s">
-        <v>7595</v>
+        <v>7596</v>
       </c>
       <c r="E1384" t="s">
         <v>7978</v>
@@ -55670,7 +55670,7 @@
         <v>6161</v>
       </c>
       <c r="D1385" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1385" t="s">
         <v>7978</v>
@@ -55693,7 +55693,7 @@
         <v>6161</v>
       </c>
       <c r="D1386" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1386" t="s">
         <v>7978</v>
@@ -55716,7 +55716,7 @@
         <v>6161</v>
       </c>
       <c r="D1387" t="s">
-        <v>7667</v>
+        <v>7668</v>
       </c>
       <c r="E1387" t="s">
         <v>7978</v>
@@ -55739,7 +55739,7 @@
         <v>6161</v>
       </c>
       <c r="D1388" t="s">
-        <v>7587</v>
+        <v>7588</v>
       </c>
       <c r="E1388" t="s">
         <v>7978</v>
@@ -55762,7 +55762,7 @@
         <v>6016</v>
       </c>
       <c r="D1389" t="s">
-        <v>7627</v>
+        <v>7628</v>
       </c>
       <c r="E1389" t="s">
         <v>7978</v>
@@ -55808,7 +55808,7 @@
         <v>6537</v>
       </c>
       <c r="D1391" t="s">
-        <v>7668</v>
+        <v>7669</v>
       </c>
       <c r="E1391" t="s">
         <v>7978</v>
@@ -55831,7 +55831,7 @@
         <v>6013</v>
       </c>
       <c r="D1392" t="s">
-        <v>7669</v>
+        <v>7670</v>
       </c>
       <c r="E1392" t="s">
         <v>7978</v>
@@ -55854,7 +55854,7 @@
         <v>5928</v>
       </c>
       <c r="D1393" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1393" t="s">
         <v>7978</v>
@@ -55923,7 +55923,7 @@
         <v>5928</v>
       </c>
       <c r="D1396" t="s">
-        <v>7670</v>
+        <v>7671</v>
       </c>
       <c r="E1396" t="s">
         <v>7978</v>
@@ -55969,7 +55969,7 @@
         <v>5928</v>
       </c>
       <c r="D1398" t="s">
-        <v>7579</v>
+        <v>7580</v>
       </c>
       <c r="E1398" t="s">
         <v>7978</v>
@@ -55992,7 +55992,7 @@
         <v>6161</v>
       </c>
       <c r="D1399" t="s">
-        <v>7574</v>
+        <v>7575</v>
       </c>
       <c r="E1399" t="s">
         <v>7978</v>
@@ -56015,7 +56015,7 @@
         <v>6161</v>
       </c>
       <c r="D1400" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1400" t="s">
         <v>7978</v>
@@ -56084,7 +56084,7 @@
         <v>6161</v>
       </c>
       <c r="D1403" t="s">
-        <v>7581</v>
+        <v>7582</v>
       </c>
       <c r="E1403" t="s">
         <v>7978</v>
@@ -56153,7 +56153,7 @@
         <v>5938</v>
       </c>
       <c r="D1406" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1406" t="s">
         <v>7978</v>
@@ -56176,7 +56176,7 @@
         <v>6161</v>
       </c>
       <c r="D1407" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1407" t="s">
         <v>7978</v>
@@ -56199,7 +56199,7 @@
         <v>6161</v>
       </c>
       <c r="D1408" t="s">
-        <v>7671</v>
+        <v>7672</v>
       </c>
       <c r="E1408" t="s">
         <v>7978</v>
@@ -56222,7 +56222,7 @@
         <v>5928</v>
       </c>
       <c r="D1409" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1409" t="s">
         <v>7978</v>
@@ -56245,7 +56245,7 @@
         <v>5938</v>
       </c>
       <c r="D1410" t="s">
-        <v>7574</v>
+        <v>7575</v>
       </c>
       <c r="E1410" t="s">
         <v>7978</v>
@@ -56268,7 +56268,7 @@
         <v>6161</v>
       </c>
       <c r="D1411" t="s">
-        <v>7672</v>
+        <v>7673</v>
       </c>
       <c r="E1411" t="s">
         <v>7978</v>
@@ -56291,7 +56291,7 @@
         <v>6161</v>
       </c>
       <c r="D1412" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1412" t="s">
         <v>7978</v>
@@ -56314,7 +56314,7 @@
         <v>6161</v>
       </c>
       <c r="D1413" t="s">
-        <v>7673</v>
+        <v>7674</v>
       </c>
       <c r="E1413" t="s">
         <v>7978</v>
@@ -56337,7 +56337,7 @@
         <v>6161</v>
       </c>
       <c r="D1414" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E1414" t="s">
         <v>7978</v>
@@ -56383,7 +56383,7 @@
         <v>6161</v>
       </c>
       <c r="D1416" t="s">
-        <v>7674</v>
+        <v>7675</v>
       </c>
       <c r="E1416" t="s">
         <v>7978</v>
@@ -56406,7 +56406,7 @@
         <v>6161</v>
       </c>
       <c r="D1417" t="s">
-        <v>7584</v>
+        <v>7585</v>
       </c>
       <c r="E1417" t="s">
         <v>7978</v>
@@ -56429,7 +56429,7 @@
         <v>6161</v>
       </c>
       <c r="D1418" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1418" t="s">
         <v>7978</v>
@@ -56498,7 +56498,7 @@
         <v>6538</v>
       </c>
       <c r="D1421" t="s">
-        <v>7619</v>
+        <v>7620</v>
       </c>
       <c r="E1421" t="s">
         <v>7978</v>
@@ -56521,7 +56521,7 @@
         <v>6161</v>
       </c>
       <c r="D1422" t="s">
-        <v>7675</v>
+        <v>7676</v>
       </c>
       <c r="E1422" t="s">
         <v>7978</v>
@@ -56544,7 +56544,7 @@
         <v>6527</v>
       </c>
       <c r="D1423" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1423" t="s">
         <v>7978</v>
@@ -56590,7 +56590,7 @@
         <v>6161</v>
       </c>
       <c r="D1425" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1425" t="s">
         <v>7978</v>
@@ -56613,7 +56613,7 @@
         <v>6538</v>
       </c>
       <c r="D1426" t="s">
-        <v>7676</v>
+        <v>7677</v>
       </c>
       <c r="E1426" t="s">
         <v>7978</v>
@@ -56659,7 +56659,7 @@
         <v>6531</v>
       </c>
       <c r="D1428" t="s">
-        <v>7677</v>
+        <v>7678</v>
       </c>
       <c r="E1428" t="s">
         <v>7978</v>
@@ -56682,7 +56682,7 @@
         <v>6161</v>
       </c>
       <c r="D1429" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1429" t="s">
         <v>7978</v>
@@ -56705,7 +56705,7 @@
         <v>6161</v>
       </c>
       <c r="D1430" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1430" t="s">
         <v>7978</v>
@@ -56728,7 +56728,7 @@
         <v>5938</v>
       </c>
       <c r="D1431" t="s">
-        <v>7678</v>
+        <v>7679</v>
       </c>
       <c r="E1431" t="s">
         <v>7978</v>
@@ -56751,7 +56751,7 @@
         <v>5938</v>
       </c>
       <c r="D1432" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1432" t="s">
         <v>7978</v>
@@ -56797,7 +56797,7 @@
         <v>5928</v>
       </c>
       <c r="D1434" t="s">
-        <v>7679</v>
+        <v>7680</v>
       </c>
       <c r="E1434" t="s">
         <v>7978</v>
@@ -56820,7 +56820,7 @@
         <v>5928</v>
       </c>
       <c r="D1435" t="s">
-        <v>7680</v>
+        <v>7681</v>
       </c>
       <c r="E1435" t="s">
         <v>7978</v>
@@ -56866,7 +56866,7 @@
         <v>5938</v>
       </c>
       <c r="D1437" t="s">
-        <v>7681</v>
+        <v>7682</v>
       </c>
       <c r="E1437" t="s">
         <v>7978</v>
@@ -56889,7 +56889,7 @@
         <v>5928</v>
       </c>
       <c r="D1438" t="s">
-        <v>7595</v>
+        <v>7596</v>
       </c>
       <c r="E1438" t="s">
         <v>7978</v>
@@ -56935,7 +56935,7 @@
         <v>6161</v>
       </c>
       <c r="D1440" t="s">
-        <v>7682</v>
+        <v>7683</v>
       </c>
       <c r="E1440" t="s">
         <v>7978</v>
@@ -56958,7 +56958,7 @@
         <v>6161</v>
       </c>
       <c r="D1441" t="s">
-        <v>7681</v>
+        <v>7682</v>
       </c>
       <c r="E1441" t="s">
         <v>7978</v>
@@ -56981,7 +56981,7 @@
         <v>5928</v>
       </c>
       <c r="D1442" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1442" t="s">
         <v>7978</v>
@@ -57027,7 +57027,7 @@
         <v>6016</v>
       </c>
       <c r="D1444" t="s">
-        <v>7586</v>
+        <v>7587</v>
       </c>
       <c r="E1444" t="s">
         <v>7978</v>
@@ -57050,7 +57050,7 @@
         <v>6523</v>
       </c>
       <c r="D1445" t="s">
-        <v>7668</v>
+        <v>7669</v>
       </c>
       <c r="E1445" t="s">
         <v>7978</v>
@@ -57073,7 +57073,7 @@
         <v>5928</v>
       </c>
       <c r="D1446" t="s">
-        <v>7579</v>
+        <v>7580</v>
       </c>
       <c r="E1446" t="s">
         <v>7978</v>
@@ -57142,7 +57142,7 @@
         <v>6161</v>
       </c>
       <c r="D1449" t="s">
-        <v>7683</v>
+        <v>7684</v>
       </c>
       <c r="E1449" t="s">
         <v>7978</v>
@@ -57165,7 +57165,7 @@
         <v>6161</v>
       </c>
       <c r="D1450" t="s">
-        <v>7684</v>
+        <v>7685</v>
       </c>
       <c r="E1450" t="s">
         <v>7978</v>
@@ -57211,7 +57211,7 @@
         <v>5938</v>
       </c>
       <c r="D1452" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1452" t="s">
         <v>7978</v>
@@ -57280,7 +57280,7 @@
         <v>5928</v>
       </c>
       <c r="D1455" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1455" t="s">
         <v>7978</v>
@@ -57326,7 +57326,7 @@
         <v>6161</v>
       </c>
       <c r="D1457" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1457" t="s">
         <v>7978</v>
@@ -57349,7 +57349,7 @@
         <v>6161</v>
       </c>
       <c r="D1458" t="s">
-        <v>7626</v>
+        <v>7627</v>
       </c>
       <c r="E1458" t="s">
         <v>7978</v>
@@ -57372,7 +57372,7 @@
         <v>6161</v>
       </c>
       <c r="D1459" t="s">
-        <v>7572</v>
+        <v>7573</v>
       </c>
       <c r="E1459" t="s">
         <v>7978</v>
@@ -57418,7 +57418,7 @@
         <v>5938</v>
       </c>
       <c r="D1461" t="s">
-        <v>7685</v>
+        <v>7686</v>
       </c>
       <c r="E1461" t="s">
         <v>7978</v>
@@ -57441,7 +57441,7 @@
         <v>6161</v>
       </c>
       <c r="D1462" t="s">
-        <v>7587</v>
+        <v>7588</v>
       </c>
       <c r="E1462" t="s">
         <v>7978</v>
@@ -57487,7 +57487,7 @@
         <v>6161</v>
       </c>
       <c r="D1464" t="s">
-        <v>7574</v>
+        <v>7575</v>
       </c>
       <c r="E1464" t="s">
         <v>7978</v>
@@ -57510,7 +57510,7 @@
         <v>6539</v>
       </c>
       <c r="D1465" t="s">
-        <v>7686</v>
+        <v>7687</v>
       </c>
       <c r="E1465" t="s">
         <v>7978</v>
@@ -57533,7 +57533,7 @@
         <v>6161</v>
       </c>
       <c r="D1466" t="s">
-        <v>7570</v>
+        <v>7571</v>
       </c>
       <c r="E1466" t="s">
         <v>7978</v>
@@ -57556,7 +57556,7 @@
         <v>5938</v>
       </c>
       <c r="D1467" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1467" t="s">
         <v>7978</v>
@@ -57602,7 +57602,7 @@
         <v>6161</v>
       </c>
       <c r="D1469" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1469" t="s">
         <v>7978</v>
@@ -57625,7 +57625,7 @@
         <v>5938</v>
       </c>
       <c r="D1470" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1470" t="s">
         <v>7978</v>
@@ -57648,7 +57648,7 @@
         <v>6161</v>
       </c>
       <c r="D1471" t="s">
-        <v>7687</v>
+        <v>7688</v>
       </c>
       <c r="E1471" t="s">
         <v>7978</v>
@@ -57671,7 +57671,7 @@
         <v>6161</v>
       </c>
       <c r="D1472" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1472" t="s">
         <v>7978</v>
@@ -57694,7 +57694,7 @@
         <v>5928</v>
       </c>
       <c r="D1473" t="s">
-        <v>7606</v>
+        <v>7607</v>
       </c>
       <c r="E1473" t="s">
         <v>7978</v>
@@ -57763,7 +57763,7 @@
         <v>6119</v>
       </c>
       <c r="D1476" t="s">
-        <v>7688</v>
+        <v>7689</v>
       </c>
       <c r="E1476" t="s">
         <v>7978</v>
@@ -57809,7 +57809,7 @@
         <v>6161</v>
       </c>
       <c r="D1478" t="s">
-        <v>7586</v>
+        <v>7587</v>
       </c>
       <c r="E1478" t="s">
         <v>7978</v>
@@ -57832,7 +57832,7 @@
         <v>5938</v>
       </c>
       <c r="D1479" t="s">
-        <v>7689</v>
+        <v>7690</v>
       </c>
       <c r="E1479" t="s">
         <v>7978</v>
@@ -57855,7 +57855,7 @@
         <v>6161</v>
       </c>
       <c r="D1480" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1480" t="s">
         <v>7978</v>
@@ -57878,7 +57878,7 @@
         <v>6161</v>
       </c>
       <c r="D1481" t="s">
-        <v>7572</v>
+        <v>7573</v>
       </c>
       <c r="E1481" t="s">
         <v>7978</v>
@@ -57901,7 +57901,7 @@
         <v>6161</v>
       </c>
       <c r="D1482" t="s">
-        <v>7585</v>
+        <v>7586</v>
       </c>
       <c r="E1482" t="s">
         <v>7978</v>
@@ -57924,7 +57924,7 @@
         <v>5938</v>
       </c>
       <c r="D1483" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1483" t="s">
         <v>7978</v>
@@ -57970,7 +57970,7 @@
         <v>6540</v>
       </c>
       <c r="D1485" t="s">
-        <v>7680</v>
+        <v>7681</v>
       </c>
       <c r="E1485" t="s">
         <v>7978</v>
@@ -58062,7 +58062,7 @@
         <v>5938</v>
       </c>
       <c r="D1489" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1489" t="s">
         <v>7978</v>
@@ -58085,7 +58085,7 @@
         <v>6161</v>
       </c>
       <c r="D1490" t="s">
-        <v>7690</v>
+        <v>7691</v>
       </c>
       <c r="E1490" t="s">
         <v>7978</v>
@@ -58177,7 +58177,7 @@
         <v>6161</v>
       </c>
       <c r="D1494" t="s">
-        <v>7567</v>
+        <v>7568</v>
       </c>
       <c r="E1494" t="s">
         <v>7978</v>
@@ -58200,7 +58200,7 @@
         <v>5928</v>
       </c>
       <c r="D1495" t="s">
-        <v>7680</v>
+        <v>7681</v>
       </c>
       <c r="E1495" t="s">
         <v>7978</v>
@@ -58223,7 +58223,7 @@
         <v>6161</v>
       </c>
       <c r="D1496" t="s">
-        <v>7691</v>
+        <v>7692</v>
       </c>
       <c r="E1496" t="s">
         <v>7978</v>
@@ -58246,7 +58246,7 @@
         <v>6161</v>
       </c>
       <c r="D1497" t="s">
-        <v>7587</v>
+        <v>7588</v>
       </c>
       <c r="E1497" t="s">
         <v>7978</v>
@@ -58269,7 +58269,7 @@
         <v>6161</v>
       </c>
       <c r="D1498" t="s">
-        <v>7692</v>
+        <v>7693</v>
       </c>
       <c r="E1498" t="s">
         <v>7978</v>
@@ -58292,7 +58292,7 @@
         <v>6161</v>
       </c>
       <c r="D1499" t="s">
-        <v>7594</v>
+        <v>7595</v>
       </c>
       <c r="E1499" t="s">
         <v>7978</v>
@@ -58315,7 +58315,7 @@
         <v>5938</v>
       </c>
       <c r="D1500" t="s">
-        <v>7693</v>
+        <v>7694</v>
       </c>
       <c r="E1500" t="s">
         <v>7978</v>
@@ -58338,7 +58338,7 @@
         <v>6161</v>
       </c>
       <c r="D1501" t="s">
-        <v>7572</v>
+        <v>7573</v>
       </c>
       <c r="E1501" t="s">
         <v>7978</v>
@@ -58361,7 +58361,7 @@
         <v>6161</v>
       </c>
       <c r="D1502" t="s">
-        <v>7571</v>
+        <v>7572</v>
       </c>
       <c r="E1502" t="s">
         <v>7978</v>
@@ -58384,7 +58384,7 @@
         <v>5915</v>
       </c>
       <c r="D1503" t="s">
-        <v>7694</v>
+        <v>7695</v>
       </c>
       <c r="E1503" t="s">
         <v>7978</v>
@@ -58430,7 +58430,7 @@
         <v>6126</v>
       </c>
       <c r="D1505" t="s">
-        <v>7640</v>
+        <v>7641</v>
       </c>
       <c r="E1505" t="s">
         <v>7978</v>
@@ -58453,7 +58453,7 @@
         <v>6161</v>
       </c>
       <c r="D1506" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1506" t="s">
         <v>7978</v>
@@ -58476,7 +58476,7 @@
         <v>5938</v>
       </c>
       <c r="D1507" t="s">
-        <v>7582</v>
+        <v>7583</v>
       </c>
       <c r="E1507" t="s">
         <v>7978</v>
@@ -58499,7 +58499,7 @@
         <v>6161</v>
       </c>
       <c r="D1508" t="s">
-        <v>7695</v>
+        <v>7696</v>
       </c>
       <c r="E1508" t="s">
         <v>7978</v>
@@ -58522,7 +58522,7 @@
         <v>5938</v>
       </c>
       <c r="D1509" t="s">
-        <v>7572</v>
+        <v>7573</v>
       </c>
       <c r="E1509" t="s">
         <v>7978</v>
@@ -58545,7 +58545,7 @@
         <v>6161</v>
       </c>
       <c r="D1510" t="s">
-        <v>7696</v>
+        <v>7697</v>
       </c>
       <c r="E1510" t="s">
         <v>7978</v>
@@ -58568,7 +58568,7 @@
         <v>6016</v>
       </c>
       <c r="D1511" t="s">
-        <v>7613</v>
+        <v>7614</v>
       </c>
       <c r="E1511" t="s">
         <v>7978</v>
@@ -58614,7 +58614,7 @@
         <v>5928</v>
       </c>
       <c r="D1513" t="s">
-        <v>7566</v>
+        <v>7567</v>
       </c>
       <c r="E1513" t="s">
         <v>7978</v>
@@ -58683,7 +58683,7 @@
         <v>5928</v>
       </c>
       <c r="D1516" t="s">
-        <v>7634</v>
+        <v>7635</v>
       </c>
       <c r="E1516" t="s">
         <v>7978</v>
@@ -58706,7 +58706,7 @@
         <v>5928</v>
       </c>
       <c r="D1517" t="s">
-        <v>7602</v>
+        <v>7603</v>
       </c>
       <c r="E1517" t="s">
         <v>7978</v>
@@ -58729,7 +58729,7 @@
         <v>6161</v>
       </c>
       <c r="D1518" t="s">
-        <v>7612</v>
+        <v>7613</v>
       </c>
       <c r="E1518" t="s">
         <v>7978</v>
@@ -58752,7 +58752,7 @@
         <v>6161</v>
       </c>
       <c r="D1519" t="s">
-        <v>7574</v>
+        <v>7575</v>
       </c>
       <c r="E1519" t="s">
         <v>7978</v>
@@ -58821,7 +58821,7 @@
         <v>6542</v>
       </c>
       <c r="D1522" t="s">
-        <v>7697</v>
+        <v>7698</v>
       </c>
       <c r="E1522" t="s">
         <v>7979</v>
@@ -58867,7 +58867,7 @@
         <v>6543</v>
       </c>
       <c r="D1524" t="s">
-        <v>7698</v>
+        <v>7699</v>
       </c>
       <c r="E1524" t="s">
         <v>7979</v>
@@ -58890,7 +58890,7 @@
         <v>6013</v>
       </c>
       <c r="D1525" t="s">
-        <v>7654</v>
+        <v>7655</v>
       </c>
       <c r="E1525" t="s">
         <v>7979</v>
@@ -58913,7 +58913,7 @@
         <v>6522</v>
       </c>
       <c r="D1526" t="s">
-        <v>7699</v>
+        <v>7700</v>
       </c>
       <c r="E1526" t="s">
         <v>7979</v>
@@ -58936,7 +58936,7 @@
         <v>6522</v>
       </c>
       <c r="D1527" t="s">
-        <v>7700</v>
+        <v>7701</v>
       </c>
       <c r="E1527" t="s">
         <v>7979</v>
@@ -58982,7 +58982,7 @@
         <v>6544</v>
       </c>
       <c r="D1529" t="s">
-        <v>7701</v>
+        <v>7702</v>
       </c>
       <c r="E1529" t="s">
         <v>7979</v>
@@ -59051,7 +59051,7 @@
         <v>6545</v>
       </c>
       <c r="D1532" t="s">
-        <v>7645</v>
+        <v>7646</v>
       </c>
       <c r="E1532" t="s">
         <v>7979</v>
@@ -59074,7 +59074,7 @@
         <v>6546</v>
       </c>
       <c r="D1533" t="s">
-        <v>7702</v>
+        <v>7703</v>
       </c>
       <c r="E1533" t="s">
         <v>7979</v>
@@ -59097,7 +59097,7 @@
         <v>6547</v>
       </c>
       <c r="D1534" t="s">
-        <v>7646</v>
+        <v>7647</v>
       </c>
       <c r="E1534" t="s">
         <v>7979</v>
@@ -59120,7 +59120,7 @@
         <v>6548</v>
       </c>
       <c r="D1535" t="s">
-        <v>7703</v>
+        <v>7704</v>
       </c>
       <c r="E1535" t="s">
         <v>7979</v>
@@ -59166,7 +59166,7 @@
         <v>6549</v>
       </c>
       <c r="D1537" t="s">
-        <v>7645</v>
+        <v>7646</v>
       </c>
       <c r="E1537" t="s">
         <v>7979</v>
@@ -59189,7 +59189,7 @@
         <v>6550</v>
       </c>
       <c r="D1538" t="s">
-        <v>7704</v>
+        <v>7705</v>
       </c>
       <c r="E1538" t="s">
         <v>7979</v>
@@ -59235,7 +59235,7 @@
         <v>6551</v>
       </c>
       <c r="D1540" t="s">
-        <v>7705</v>
+        <v>7706</v>
       </c>
       <c r="E1540" t="s">
         <v>7979</v>
@@ -59281,7 +59281,7 @@
         <v>6553</v>
       </c>
       <c r="D1542" t="s">
-        <v>7706</v>
+        <v>7707</v>
       </c>
       <c r="E1542" t="s">
         <v>7979</v>
@@ -59304,7 +59304,7 @@
         <v>6554</v>
       </c>
       <c r="D1543" t="s">
-        <v>7707</v>
+        <v>7708</v>
       </c>
       <c r="E1543" t="s">
         <v>7979</v>
@@ -59396,7 +59396,7 @@
         <v>6556</v>
       </c>
       <c r="D1547" t="s">
-        <v>7708</v>
+        <v>7709</v>
       </c>
       <c r="E1547" t="s">
         <v>7979</v>
@@ -59419,7 +59419,7 @@
         <v>6557</v>
       </c>
       <c r="D1548" t="s">
-        <v>7645</v>
+        <v>7646</v>
       </c>
       <c r="E1548" t="s">
         <v>7979</v>
@@ -59511,7 +59511,7 @@
         <v>6265</v>
       </c>
       <c r="D1552" t="s">
-        <v>7709</v>
+        <v>7710</v>
       </c>
       <c r="E1552" t="s">
         <v>7979</v>
@@ -59534,7 +59534,7 @@
         <v>6559</v>
       </c>
       <c r="D1553" t="s">
-        <v>7710</v>
+        <v>7407</v>
       </c>
       <c r="E1553" t="s">
         <v>7979</v>
@@ -59810,7 +59810,7 @@
         <v>6041</v>
       </c>
       <c r="D1565" t="s">
-        <v>7688</v>
+        <v>7689</v>
       </c>
       <c r="E1565" t="s">
         <v>7979</v>
@@ -59902,7 +59902,7 @@
         <v>6565</v>
       </c>
       <c r="D1569" t="s">
-        <v>7614</v>
+        <v>7615</v>
       </c>
       <c r="E1569" t="s">
         <v>7979</v>
@@ -60109,7 +60109,7 @@
         <v>6547</v>
       </c>
       <c r="D1578" t="s">
-        <v>7646</v>
+        <v>7647</v>
       </c>
       <c r="E1578" t="s">
         <v>7979</v>
@@ -60339,7 +60339,7 @@
         <v>6042</v>
       </c>
       <c r="D1588" t="s">
-        <v>7581</v>
+        <v>7582</v>
       </c>
       <c r="E1588" t="s">
         <v>7979</v>
@@ -60362,7 +60362,7 @@
         <v>6572</v>
       </c>
       <c r="D1589" t="s">
-        <v>7688</v>
+        <v>7689</v>
       </c>
       <c r="E1589" t="s">
         <v>7979</v>
@@ -60500,7 +60500,7 @@
         <v>6557</v>
       </c>
       <c r="D1595" t="s">
-        <v>7710</v>
+        <v>7407</v>
       </c>
       <c r="E1595" t="s">
         <v>7979</v>
@@ -60569,7 +60569,7 @@
         <v>6577</v>
       </c>
       <c r="D1598" t="s">
-        <v>7703</v>
+        <v>7704</v>
       </c>
       <c r="E1598" t="s">
         <v>7979</v>
@@ -60615,7 +60615,7 @@
         <v>6578</v>
       </c>
       <c r="D1600" t="s">
-        <v>7705</v>
+        <v>7706</v>
       </c>
       <c r="E1600" t="s">
         <v>7979</v>
@@ -60638,7 +60638,7 @@
         <v>6579</v>
       </c>
       <c r="D1601" t="s">
-        <v>7594</v>
+        <v>7595</v>
       </c>
       <c r="E1601" t="s">
         <v>7979</v>
@@ -60684,7 +60684,7 @@
         <v>6581</v>
       </c>
       <c r="D1603" t="s">
-        <v>7688</v>
+        <v>7689</v>
       </c>
       <c r="E1603" t="s">
         <v>7979</v>
@@ -61167,7 +61167,7 @@
         <v>6595</v>
       </c>
       <c r="D1624" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E1624" t="s">
         <v>7979</v>
@@ -61305,7 +61305,7 @@
         <v>6161</v>
       </c>
       <c r="D1630" t="s">
-        <v>7653</v>
+        <v>7654</v>
       </c>
       <c r="E1630" t="s">
         <v>7979</v>
@@ -61443,7 +61443,7 @@
         <v>6600</v>
       </c>
       <c r="D1636" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1636" t="s">
         <v>7979</v>
@@ -61719,7 +61719,7 @@
         <v>6605</v>
       </c>
       <c r="D1648" t="s">
-        <v>7685</v>
+        <v>7686</v>
       </c>
       <c r="E1648" t="s">
         <v>7979</v>
@@ -62041,7 +62041,7 @@
         <v>6612</v>
       </c>
       <c r="D1662" t="s">
-        <v>7689</v>
+        <v>7690</v>
       </c>
       <c r="E1662" t="s">
         <v>7979</v>
@@ -62156,7 +62156,7 @@
         <v>6614</v>
       </c>
       <c r="D1667" t="s">
-        <v>7614</v>
+        <v>7615</v>
       </c>
       <c r="E1667" t="s">
         <v>7979</v>
@@ -62524,7 +62524,7 @@
         <v>6210</v>
       </c>
       <c r="D1683" t="s">
-        <v>7703</v>
+        <v>7704</v>
       </c>
       <c r="E1683" t="s">
         <v>7979</v>
@@ -62547,7 +62547,7 @@
         <v>6558</v>
       </c>
       <c r="D1684" t="s">
-        <v>7614</v>
+        <v>7615</v>
       </c>
       <c r="E1684" t="s">
         <v>7979</v>
@@ -62731,7 +62731,7 @@
         <v>6612</v>
       </c>
       <c r="D1692" t="s">
-        <v>7710</v>
+        <v>7407</v>
       </c>
       <c r="E1692" t="s">
         <v>7979</v>
@@ -62754,7 +62754,7 @@
         <v>6620</v>
       </c>
       <c r="D1693" t="s">
-        <v>7710</v>
+        <v>7407</v>
       </c>
       <c r="E1693" t="s">
         <v>7979</v>
@@ -62823,7 +62823,7 @@
         <v>6622</v>
       </c>
       <c r="D1696" t="s">
-        <v>7646</v>
+        <v>7647</v>
       </c>
       <c r="E1696" t="s">
         <v>7979</v>
@@ -63053,7 +63053,7 @@
         <v>6550</v>
       </c>
       <c r="D1706" t="s">
-        <v>7614</v>
+        <v>7615</v>
       </c>
       <c r="E1706" t="s">
         <v>7979</v>
@@ -63191,7 +63191,7 @@
         <v>5950</v>
       </c>
       <c r="D1712" t="s">
-        <v>7572</v>
+        <v>7573</v>
       </c>
       <c r="E1712" t="s">
         <v>7979</v>
@@ -63697,7 +63697,7 @@
         <v>6338</v>
       </c>
       <c r="D1734" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1734" t="s">
         <v>7979</v>
@@ -65887,7 +65887,7 @@
         <v>5990</v>
       </c>
       <c r="D1836" t="s">
-        <v>7703</v>
+        <v>7704</v>
       </c>
       <c r="E1836" t="s">
         <v>7985</v>
@@ -68038,7 +68038,7 @@
         <v>6616</v>
       </c>
       <c r="D1941" t="s">
-        <v>7614</v>
+        <v>7615</v>
       </c>
       <c r="E1941" t="s">
         <v>7987</v>
@@ -68213,7 +68213,7 @@
         <v>5917</v>
       </c>
       <c r="D1949" t="s">
-        <v>7663</v>
+        <v>7664</v>
       </c>
       <c r="E1949" t="s">
         <v>7987</v>
@@ -68428,7 +68428,7 @@
         <v>5977</v>
       </c>
       <c r="D1959" t="s">
-        <v>7591</v>
+        <v>7592</v>
       </c>
       <c r="E1959" t="s">
         <v>7989</v>
@@ -68976,7 +68976,7 @@
         <v>6155</v>
       </c>
       <c r="D1984" t="s">
-        <v>7578</v>
+        <v>7579</v>
       </c>
       <c r="E1984" t="s">
         <v>7992</v>
@@ -69203,7 +69203,7 @@
         <v>6013</v>
       </c>
       <c r="D1994" t="s">
-        <v>7580</v>
+        <v>7581</v>
       </c>
       <c r="E1994" t="s">
         <v>7994</v>
@@ -69493,7 +69493,7 @@
         <v>5938</v>
       </c>
       <c r="D2007" t="s">
-        <v>7614</v>
+        <v>7615</v>
       </c>
       <c r="E2007" t="s">
         <v>7995</v>
@@ -70633,7 +70633,7 @@
         <v>6770</v>
       </c>
       <c r="D2061" t="s">
-        <v>7668</v>
+        <v>7669</v>
       </c>
       <c r="E2061" t="s">
         <v>7996</v>
@@ -71706,7 +71706,7 @@
         <v>6541</v>
       </c>
       <c r="D2113" t="s">
-        <v>7705</v>
+        <v>7706</v>
       </c>
       <c r="E2113" t="s">
         <v>8002</v>
@@ -73908,7 +73908,7 @@
         <v>6846</v>
       </c>
       <c r="D2218" t="s">
-        <v>7591</v>
+        <v>7592</v>
       </c>
       <c r="E2218" t="s">
         <v>8006</v>
@@ -74283,7 +74283,7 @@
         <v>6885</v>
       </c>
       <c r="D2236" t="s">
-        <v>7591</v>
+        <v>7592</v>
       </c>
       <c r="E2236" t="s">
         <v>8008</v>
@@ -74323,7 +74323,7 @@
         <v>6887</v>
       </c>
       <c r="D2238" t="s">
-        <v>7580</v>
+        <v>7581</v>
       </c>
       <c r="E2238" t="s">
         <v>8008</v>
@@ -74839,7 +74839,7 @@
         <v>6692</v>
       </c>
       <c r="D2262" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E2262" t="s">
         <v>8010</v>
@@ -74862,7 +74862,7 @@
         <v>6895</v>
       </c>
       <c r="D2263" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E2263" t="s">
         <v>8010</v>
@@ -74931,7 +74931,7 @@
         <v>6898</v>
       </c>
       <c r="D2266" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E2266" t="s">
         <v>8010</v>
@@ -75023,7 +75023,7 @@
         <v>5909</v>
       </c>
       <c r="D2270" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E2270" t="s">
         <v>8010</v>
@@ -75046,7 +75046,7 @@
         <v>6105</v>
       </c>
       <c r="D2271" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E2271" t="s">
         <v>8010</v>
@@ -75069,7 +75069,7 @@
         <v>6900</v>
       </c>
       <c r="D2272" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E2272" t="s">
         <v>8010</v>
@@ -75207,7 +75207,7 @@
         <v>6902</v>
       </c>
       <c r="D2278" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E2278" t="s">
         <v>8010</v>
@@ -75276,7 +75276,7 @@
         <v>5915</v>
       </c>
       <c r="D2281" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E2281" t="s">
         <v>8010</v>
@@ -76576,7 +76576,7 @@
         <v>6161</v>
       </c>
       <c r="D2340" t="s">
-        <v>7580</v>
+        <v>7581</v>
       </c>
       <c r="E2340" t="s">
         <v>8011</v>
@@ -79056,7 +79056,7 @@
         <v>6955</v>
       </c>
       <c r="D2455" t="s">
-        <v>7634</v>
+        <v>7635</v>
       </c>
       <c r="E2455" t="s">
         <v>8014</v>
@@ -79811,7 +79811,7 @@
         <v>6126</v>
       </c>
       <c r="D2489" t="s">
-        <v>7703</v>
+        <v>7704</v>
       </c>
       <c r="E2489" t="s">
         <v>8017</v>
@@ -81857,7 +81857,7 @@
         <v>5990</v>
       </c>
       <c r="D2588" t="s">
-        <v>7701</v>
+        <v>7702</v>
       </c>
       <c r="E2588" t="s">
         <v>8022</v>
@@ -84483,7 +84483,7 @@
         <v>6504</v>
       </c>
       <c r="D2707" t="s">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="E2707" t="s">
         <v>8026</v>
@@ -85474,7 +85474,7 @@
         <v>7039</v>
       </c>
       <c r="D2754" t="s">
-        <v>7591</v>
+        <v>7592</v>
       </c>
       <c r="E2754" t="s">
         <v>8028</v>
@@ -87035,7 +87035,7 @@
         <v>7089</v>
       </c>
       <c r="D2828" t="s">
-        <v>7666</v>
+        <v>7667</v>
       </c>
       <c r="E2828" t="s">
         <v>8032</v>
@@ -87115,7 +87115,7 @@
         <v>7082</v>
       </c>
       <c r="D2832" t="s">
-        <v>7634</v>
+        <v>7635</v>
       </c>
       <c r="E2832" t="s">
         <v>8032</v>
@@ -89668,7 +89668,7 @@
         <v>7163</v>
       </c>
       <c r="D2955" t="s">
-        <v>7565</v>
+        <v>7566</v>
       </c>
       <c r="E2955" t="s">
         <v>8041</v>

</xml_diff>